<commit_message>
Atualiza ajustes de competicoes
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -583,13 +583,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>66.86</v>
+        <v>66.85986328125</v>
       </c>
       <c r="H2">
-        <v>54.6</v>
+        <v>54.60009765625</v>
       </c>
       <c r="I2">
-        <v>12.26</v>
+        <v>12.259765625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -618,10 +618,10 @@
         <v>49</v>
       </c>
       <c r="H3">
-        <v>47.86</v>
+        <v>47.860107421875</v>
       </c>
       <c r="I3">
-        <v>1.140000000000001</v>
+        <v>1.139892578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -647,13 +647,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>54.6</v>
+        <v>54.60009765625</v>
       </c>
       <c r="H4">
-        <v>66.86</v>
+        <v>66.85986328125</v>
       </c>
       <c r="I4">
-        <v>-12.26</v>
+        <v>-12.259765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>47.86</v>
+        <v>47.860107421875</v>
       </c>
       <c r="H5">
         <v>49</v>
       </c>
       <c r="I5">
-        <v>-1.140000000000001</v>
+        <v>-1.139892578125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -753,13 +753,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>84.86</v>
+        <v>84.85986328125</v>
       </c>
       <c r="H2">
-        <v>49.76</v>
+        <v>49.760009765625</v>
       </c>
       <c r="I2">
-        <v>35.1</v>
+        <v>35.099853515625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -785,13 +785,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>72.7</v>
+        <v>72.7001953125</v>
       </c>
       <c r="H3">
-        <v>47.86</v>
+        <v>47.860107421875</v>
       </c>
       <c r="I3">
-        <v>24.84</v>
+        <v>24.840087890625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -817,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>49.76</v>
+        <v>49.760009765625</v>
       </c>
       <c r="H4">
-        <v>84.86</v>
+        <v>84.85986328125</v>
       </c>
       <c r="I4">
-        <v>-35.1</v>
+        <v>-35.099853515625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -849,13 +849,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>47.86</v>
+        <v>47.860107421875</v>
       </c>
       <c r="H5">
-        <v>72.7</v>
+        <v>72.7001953125</v>
       </c>
       <c r="I5">
-        <v>-24.84</v>
+        <v>-24.840087890625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>74.06</v>
+        <v>74.06005859375</v>
       </c>
       <c r="H2">
-        <v>61.56</v>
+        <v>61.56005859375</v>
       </c>
       <c r="I2">
         <v>12.5</v>
@@ -955,13 +955,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>72.86</v>
+        <v>72.85986328125</v>
       </c>
       <c r="H3">
-        <v>60.16</v>
+        <v>60.159912109375</v>
       </c>
       <c r="I3">
-        <v>12.7</v>
+        <v>12.699951171875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,10 +987,10 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>61.56</v>
+        <v>61.56005859375</v>
       </c>
       <c r="H4">
-        <v>74.06</v>
+        <v>74.06005859375</v>
       </c>
       <c r="I4">
         <v>-12.5</v>
@@ -1019,13 +1019,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>60.16</v>
+        <v>60.159912109375</v>
       </c>
       <c r="H5">
-        <v>72.86</v>
+        <v>72.85986328125</v>
       </c>
       <c r="I5">
-        <v>-12.7</v>
+        <v>-12.699951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1093,13 +1093,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>73.95999999999999</v>
+        <v>73.9599609375</v>
       </c>
       <c r="H2">
-        <v>53.66</v>
+        <v>53.659912109375</v>
       </c>
       <c r="I2">
-        <v>20.3</v>
+        <v>20.300048828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1125,13 +1125,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>68.06</v>
+        <v>68.06005859375</v>
       </c>
       <c r="H3">
-        <v>64.7</v>
+        <v>64.7001953125</v>
       </c>
       <c r="I3">
-        <v>3.359999999999999</v>
+        <v>3.35986328125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1157,13 +1157,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>64.7</v>
+        <v>64.7001953125</v>
       </c>
       <c r="H4">
-        <v>68.06</v>
+        <v>68.06005859375</v>
       </c>
       <c r="I4">
-        <v>-3.359999999999999</v>
+        <v>-3.35986328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1189,13 +1189,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>53.66</v>
+        <v>53.659912109375</v>
       </c>
       <c r="H5">
-        <v>73.95999999999999</v>
+        <v>73.9599609375</v>
       </c>
       <c r="I5">
-        <v>-20.3</v>
+        <v>-20.300048828125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>84.26000000000001</v>
+        <v>84.259765625</v>
       </c>
       <c r="H2">
-        <v>63.9</v>
+        <v>63.89990234375</v>
       </c>
       <c r="I2">
-        <v>20.36000000000001</v>
+        <v>20.35986328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>72.45</v>
+        <v>72.4501953125</v>
       </c>
       <c r="H3">
-        <v>54.16</v>
+        <v>54.159912109375</v>
       </c>
       <c r="I3">
-        <v>18.29000000000001</v>
+        <v>18.290283203125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1327,13 +1327,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>63.9</v>
+        <v>63.89990234375</v>
       </c>
       <c r="H4">
-        <v>84.26000000000001</v>
+        <v>84.259765625</v>
       </c>
       <c r="I4">
-        <v>-20.36000000000001</v>
+        <v>-20.35986328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>54.16</v>
+        <v>54.159912109375</v>
       </c>
       <c r="H5">
-        <v>72.45</v>
+        <v>72.4501953125</v>
       </c>
       <c r="I5">
-        <v>-18.29000000000001</v>
+        <v>-18.290283203125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1433,13 +1433,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>62.56</v>
+        <v>62.56005859375</v>
       </c>
       <c r="H2">
-        <v>38.26</v>
+        <v>38.260009765625</v>
       </c>
       <c r="I2">
-        <v>24.3</v>
+        <v>24.300048828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>60.2</v>
+        <v>60.199951171875</v>
       </c>
       <c r="H3">
         <v>59.25</v>
       </c>
       <c r="I3">
-        <v>0.9500000000000028</v>
+        <v>0.949951171875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1500,10 +1500,10 @@
         <v>59.25</v>
       </c>
       <c r="H4">
-        <v>60.2</v>
+        <v>60.199951171875</v>
       </c>
       <c r="I4">
-        <v>-0.9500000000000028</v>
+        <v>-0.949951171875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1529,13 +1529,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>38.26</v>
+        <v>38.260009765625</v>
       </c>
       <c r="H5">
-        <v>62.56</v>
+        <v>62.56005859375</v>
       </c>
       <c r="I5">
-        <v>-24.3</v>
+        <v>-24.300048828125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>73.76000000000001</v>
+        <v>73.759765625</v>
       </c>
       <c r="H2">
-        <v>57.6</v>
+        <v>57.60009765625</v>
       </c>
       <c r="I2">
-        <v>16.16</v>
+        <v>16.15966796875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>61.96</v>
+        <v>61.9599609375</v>
       </c>
       <c r="H3">
-        <v>54.1</v>
+        <v>54.10009765625</v>
       </c>
       <c r="I3">
-        <v>7.859999999999999</v>
+        <v>7.85986328125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1667,13 +1667,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>57.6</v>
+        <v>57.60009765625</v>
       </c>
       <c r="H4">
-        <v>73.76000000000001</v>
+        <v>73.759765625</v>
       </c>
       <c r="I4">
-        <v>-16.16</v>
+        <v>-16.15966796875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1699,13 +1699,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>54.1</v>
+        <v>54.10009765625</v>
       </c>
       <c r="H5">
-        <v>61.96</v>
+        <v>61.9599609375</v>
       </c>
       <c r="I5">
-        <v>-7.859999999999999</v>
+        <v>-7.85986328125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1773,13 +1773,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>68.06</v>
+        <v>68.06005859375</v>
       </c>
       <c r="H2">
-        <v>58.96</v>
+        <v>58.9599609375</v>
       </c>
       <c r="I2">
-        <v>9.100000000000001</v>
+        <v>9.10009765625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>57.45</v>
+        <v>57.449951171875</v>
       </c>
       <c r="H3">
-        <v>42.96</v>
+        <v>42.9599609375</v>
       </c>
       <c r="I3">
-        <v>14.49</v>
+        <v>14.489990234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>58.96</v>
+        <v>58.9599609375</v>
       </c>
       <c r="H4">
-        <v>68.06</v>
+        <v>68.06005859375</v>
       </c>
       <c r="I4">
-        <v>-9.100000000000001</v>
+        <v>-9.10009765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1869,13 +1869,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>42.96</v>
+        <v>42.9599609375</v>
       </c>
       <c r="H5">
-        <v>57.45</v>
+        <v>57.449951171875</v>
       </c>
       <c r="I5">
-        <v>-14.49</v>
+        <v>-14.489990234375</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza datasets das competicoes
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -59,12 +59,12 @@
     <t>Tatols Beants F.C</t>
   </si>
   <si>
+    <t>JUV. KP</t>
+  </si>
+  <si>
     <t>SERGRILLO</t>
   </si>
   <si>
-    <t>JUV. KP</t>
-  </si>
-  <si>
     <t>JV5 Tricolor Gaúcho</t>
   </si>
   <si>
@@ -74,15 +74,15 @@
     <t>S.E.R. GRILLO</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>Dom Camillo68</t>
   </si>
   <si>
     <t>Máquina Laranjja</t>
   </si>
   <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
@@ -107,24 +107,24 @@
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
+    <t>FBC Colorado</t>
+  </si>
+  <si>
     <t>Grêmio imortal 36</t>
   </si>
   <si>
-    <t>FBC Colorado</t>
-  </si>
-  <si>
     <t>Grupo E</t>
   </si>
   <si>
     <t>Paulo Virgili FC</t>
   </si>
   <si>
+    <t>Fedato Futebol Clube</t>
+  </si>
+  <si>
     <t>KillerColorado</t>
   </si>
   <si>
-    <t>Fedato Futebol Clube</t>
-  </si>
-  <si>
     <t>FÚRIA LEON</t>
   </si>
   <si>
@@ -137,24 +137,24 @@
     <t>DM Studio</t>
   </si>
   <si>
+    <t>AZURRA82</t>
+  </si>
+  <si>
     <t>Rolo Compressor ZN</t>
   </si>
   <si>
-    <t>AZURRA82</t>
-  </si>
-  <si>
     <t>Grupo G</t>
   </si>
   <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
   </si>
   <si>
+    <t>Grêmio imortal 37</t>
+  </si>
+  <si>
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
-    <t>Grêmio imortal 37</t>
-  </si>
-  <si>
     <t>A Lenda Super Vascão f.c</t>
   </si>
   <si>
@@ -164,13 +164,13 @@
     <t>Texas Club 2026</t>
   </si>
   <si>
+    <t>Super Vasco f.c</t>
+  </si>
+  <si>
     <t>Gremiomaniasm</t>
   </si>
   <si>
     <t>TEAM LOPES 99</t>
-  </si>
-  <si>
-    <t>Super Vasco f.c</t>
   </si>
 </sst>
 </file>
@@ -571,10 +571,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>66.85986328125</v>
+        <v>117.20986328125</v>
       </c>
       <c r="H2">
-        <v>54.60009765625</v>
+        <v>64.60009765625</v>
       </c>
       <c r="I2">
-        <v>12.259765625</v>
+        <v>52.60976562499999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>49</v>
+        <v>123.80009765625</v>
       </c>
       <c r="H3">
-        <v>47.860107421875</v>
+        <v>119.65986328125</v>
       </c>
       <c r="I3">
-        <v>1.139892578125</v>
+        <v>4.140234375000006</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -635,10 +635,10 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -647,13 +647,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>54.60009765625</v>
+        <v>59</v>
       </c>
       <c r="H4">
-        <v>66.85986328125</v>
+        <v>98.21010742187499</v>
       </c>
       <c r="I4">
-        <v>-12.259765625</v>
+        <v>-39.21010742187499</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -676,16 +676,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>47.860107421875</v>
+        <v>100.660107421875</v>
       </c>
       <c r="H5">
-        <v>49</v>
+        <v>118.2</v>
       </c>
       <c r="I5">
-        <v>-1.139892578125</v>
+        <v>-17.53989257812501</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>84.85986328125</v>
+        <v>130.00986328125</v>
       </c>
       <c r="H2">
-        <v>49.760009765625</v>
+        <v>65.460009765625</v>
       </c>
       <c r="I2">
-        <v>35.099853515625</v>
+        <v>64.549853515625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>72.7001953125</v>
+        <v>97.26010742187501</v>
       </c>
       <c r="H3">
-        <v>47.860107421875</v>
+        <v>111.4001953125</v>
       </c>
       <c r="I3">
-        <v>24.840087890625</v>
+        <v>-14.140087890625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -805,10 +805,10 @@
         <v>18</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -817,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>49.760009765625</v>
+        <v>88.4001953125</v>
       </c>
       <c r="H4">
-        <v>84.85986328125</v>
+        <v>93.01010742187501</v>
       </c>
       <c r="I4">
-        <v>-35.099853515625</v>
+        <v>-4.609912109375003</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>47.860107421875</v>
+        <v>88.460009765625</v>
       </c>
       <c r="H5">
-        <v>72.7001953125</v>
+        <v>134.25986328125</v>
       </c>
       <c r="I5">
-        <v>-24.840087890625</v>
+        <v>-45.799853515625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -911,10 +911,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>74.06005859375</v>
+        <v>157.61005859375</v>
       </c>
       <c r="H2">
-        <v>61.56005859375</v>
+        <v>108.51005859375</v>
       </c>
       <c r="I2">
-        <v>12.5</v>
+        <v>49.10000000000001</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>72.85986328125</v>
+        <v>119.80986328125</v>
       </c>
       <c r="H3">
-        <v>60.159912109375</v>
+        <v>143.709912109375</v>
       </c>
       <c r="I3">
-        <v>12.699951171875</v>
+        <v>-23.90004882812501</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -975,10 +975,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -987,13 +987,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>61.56005859375</v>
+        <v>103.26005859375</v>
       </c>
       <c r="H4">
-        <v>74.06005859375</v>
+        <v>100.16005859375</v>
       </c>
       <c r="I4">
-        <v>-12.5</v>
+        <v>3.100000000000009</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1016,16 +1016,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>60.159912109375</v>
+        <v>86.25991210937499</v>
       </c>
       <c r="H5">
-        <v>72.85986328125</v>
+        <v>114.55986328125</v>
       </c>
       <c r="I5">
-        <v>-12.699951171875</v>
+        <v>-28.29995117187501</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1081,10 +1081,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1093,13 +1093,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>73.9599609375</v>
+        <v>139.3599609375</v>
       </c>
       <c r="H2">
-        <v>53.659912109375</v>
+        <v>111.959912109375</v>
       </c>
       <c r="I2">
-        <v>20.300048828125</v>
+        <v>27.40004882812501</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1122,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>68.06005859375</v>
+        <v>126.36005859375</v>
       </c>
       <c r="H3">
-        <v>64.7001953125</v>
+        <v>130.1001953125</v>
       </c>
       <c r="I3">
-        <v>3.35986328125</v>
+        <v>-3.740136718750009</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1145,10 +1145,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1157,13 +1157,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>64.7001953125</v>
+        <v>103.459912109375</v>
       </c>
       <c r="H4">
-        <v>68.06005859375</v>
+        <v>109.6599609375</v>
       </c>
       <c r="I4">
-        <v>-3.35986328125</v>
+        <v>-6.200048828125006</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1186,16 +1186,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>53.659912109375</v>
+        <v>100.4001953125</v>
       </c>
       <c r="H5">
-        <v>73.9599609375</v>
+        <v>117.86005859375</v>
       </c>
       <c r="I5">
-        <v>-20.300048828125</v>
+        <v>-17.45986328124999</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1260,16 +1260,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>84.259765625</v>
+        <v>134.559765625</v>
       </c>
       <c r="H2">
-        <v>63.89990234375</v>
+        <v>123.84990234375</v>
       </c>
       <c r="I2">
-        <v>20.35986328125</v>
+        <v>10.70986328125001</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1292,16 +1292,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>72.4501953125</v>
+        <v>127.44990234375</v>
       </c>
       <c r="H3">
-        <v>54.159912109375</v>
+        <v>136.159765625</v>
       </c>
       <c r="I3">
-        <v>18.290283203125</v>
+        <v>-8.709863281250009</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1327,13 +1327,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>63.89990234375</v>
+        <v>124.3501953125</v>
       </c>
       <c r="H4">
-        <v>84.259765625</v>
+        <v>117.709912109375</v>
       </c>
       <c r="I4">
-        <v>-20.35986328125</v>
+        <v>6.640283203125009</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1347,10 +1347,10 @@
         <v>34</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1359,13 +1359,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>54.159912109375</v>
+        <v>114.109912109375</v>
       </c>
       <c r="H5">
-        <v>72.4501953125</v>
+        <v>122.7501953125</v>
       </c>
       <c r="I5">
-        <v>-18.290283203125</v>
+        <v>-8.640283203124994</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1421,10 +1421,10 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1433,13 +1433,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>62.56005859375</v>
+        <v>118.46005859375</v>
       </c>
       <c r="H2">
-        <v>38.260009765625</v>
+        <v>84.16000976562501</v>
       </c>
       <c r="I2">
-        <v>24.300048828125</v>
+        <v>34.300048828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1462,16 +1462,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>60.199951171875</v>
+        <v>106.099951171875</v>
       </c>
       <c r="H3">
-        <v>59.25</v>
+        <v>115.15</v>
       </c>
       <c r="I3">
-        <v>0.949951171875</v>
+        <v>-9.050048828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1485,10 +1485,10 @@
         <v>38</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1497,13 +1497,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>59.25</v>
+        <v>104.810009765625</v>
       </c>
       <c r="H4">
-        <v>60.199951171875</v>
+        <v>100.36005859375</v>
       </c>
       <c r="I4">
-        <v>-0.949951171875</v>
+        <v>4.449951171875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1526,16 +1526,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>38.260009765625</v>
+        <v>97.05</v>
       </c>
       <c r="H5">
-        <v>62.56005859375</v>
+        <v>126.749951171875</v>
       </c>
       <c r="I5">
-        <v>-24.300048828125</v>
+        <v>-29.699951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,10 +1591,10 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>73.759765625</v>
+        <v>127.659765625</v>
       </c>
       <c r="H2">
-        <v>57.60009765625</v>
+        <v>100.10009765625</v>
       </c>
       <c r="I2">
-        <v>16.15966796875</v>
+        <v>27.55966796875001</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1632,16 +1632,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>61.9599609375</v>
+        <v>137.20009765625</v>
       </c>
       <c r="H3">
-        <v>54.10009765625</v>
+        <v>139.259765625</v>
       </c>
       <c r="I3">
-        <v>7.85986328125</v>
+        <v>-2.059667968750006</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1655,10 +1655,10 @@
         <v>43</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1667,13 +1667,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>57.60009765625</v>
+        <v>104.4599609375</v>
       </c>
       <c r="H4">
-        <v>73.759765625</v>
+        <v>108.00009765625</v>
       </c>
       <c r="I4">
-        <v>-16.15966796875</v>
+        <v>-3.540136718750006</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>54.10009765625</v>
+        <v>119.60009765625</v>
       </c>
       <c r="H5">
-        <v>61.9599609375</v>
+        <v>141.5599609375</v>
       </c>
       <c r="I5">
-        <v>-7.85986328125</v>
+        <v>-21.95986328124999</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1761,10 +1761,10 @@
         <v>46</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1773,13 +1773,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>68.06005859375</v>
+        <v>109.76005859375</v>
       </c>
       <c r="H2">
-        <v>58.9599609375</v>
+        <v>94.7099609375</v>
       </c>
       <c r="I2">
-        <v>9.10009765625</v>
+        <v>15.05009765625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>57.449951171875</v>
+        <v>105.3599609375</v>
       </c>
       <c r="H3">
-        <v>42.9599609375</v>
+        <v>96.249951171875</v>
       </c>
       <c r="I3">
-        <v>14.489990234375</v>
+        <v>9.110009765625009</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1825,10 +1825,10 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1837,13 +1837,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>58.9599609375</v>
+        <v>93.199951171875</v>
       </c>
       <c r="H4">
-        <v>68.06005859375</v>
+        <v>84.6599609375</v>
       </c>
       <c r="I4">
-        <v>-9.10009765625</v>
+        <v>8.539990234374997</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1866,16 +1866,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>42.9599609375</v>
+        <v>97.7599609375</v>
       </c>
       <c r="H5">
-        <v>57.449951171875</v>
+        <v>130.46005859375</v>
       </c>
       <c r="I5">
-        <v>-14.489990234375</v>
+        <v>-32.70009765625001</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza datasets (exceto Copa Leon)
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -583,13 +583,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>159.55986328125</v>
+        <v>159.56005859375</v>
       </c>
       <c r="H2">
-        <v>91.03009765625001</v>
+        <v>91.030029296875</v>
       </c>
       <c r="I2">
-        <v>68.52976562499998</v>
+        <v>68.530029296875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -615,13 +615,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>140.18009765625</v>
+        <v>140.18017578125</v>
       </c>
       <c r="H3">
-        <v>139.03986328125</v>
+        <v>139.0400390625</v>
       </c>
       <c r="I3">
-        <v>1.140234374999977</v>
+        <v>1.14013671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -647,13 +647,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>85.43000000000001</v>
+        <v>85.429931640625</v>
       </c>
       <c r="H4">
-        <v>140.560107421875</v>
+        <v>140.560302734375</v>
       </c>
       <c r="I4">
-        <v>-55.13010742187498</v>
+        <v>-55.13037109375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>120.040107421875</v>
+        <v>120.040283203125</v>
       </c>
       <c r="H5">
-        <v>134.58</v>
+        <v>134.580078125</v>
       </c>
       <c r="I5">
-        <v>-14.53989257812498</v>
+        <v>-14.539794921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -753,13 +753,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>164.30986328125</v>
+        <v>164.31005859375</v>
       </c>
       <c r="H2">
-        <v>114.340009765625</v>
+        <v>114.340087890625</v>
       </c>
       <c r="I2">
-        <v>49.96985351562499</v>
+        <v>49.969970703125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -785,13 +785,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>137.2801953125</v>
+        <v>137.2802734375</v>
       </c>
       <c r="H3">
-        <v>127.310107421875</v>
+        <v>127.310302734375</v>
       </c>
       <c r="I3">
-        <v>9.970087890624981</v>
+        <v>9.969970703125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -817,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>129.740107421875</v>
+        <v>129.739990234375</v>
       </c>
       <c r="H4">
-        <v>150.1801953125</v>
+        <v>150.18017578125</v>
       </c>
       <c r="I4">
-        <v>-20.44008789062502</v>
+        <v>-20.440185546875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -849,13 +849,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>127.240009765625</v>
+        <v>127.239990234375</v>
       </c>
       <c r="H5">
-        <v>166.73986328125</v>
+        <v>166.73974609375</v>
       </c>
       <c r="I5">
-        <v>-39.49985351562499</v>
+        <v>-39.499755859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>167.84005859375</v>
+        <v>167.83984375</v>
       </c>
       <c r="H2">
-        <v>126.71005859375</v>
+        <v>126.7099609375</v>
       </c>
       <c r="I2">
-        <v>41.13</v>
+        <v>41.1298828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -955,13 +955,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>143.74005859375</v>
+        <v>143.740234375</v>
       </c>
       <c r="H3">
-        <v>138.64005859375</v>
+        <v>138.64013671875</v>
       </c>
       <c r="I3">
-        <v>5.100000000000023</v>
+        <v>5.10009765625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,13 +987,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>138.00986328125</v>
+        <v>138.009765625</v>
       </c>
       <c r="H4">
-        <v>153.939912109375</v>
+        <v>153.939697265625</v>
       </c>
       <c r="I4">
-        <v>-15.930048828125</v>
+        <v>-15.929931640625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1019,13 +1019,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>124.739912109375</v>
+        <v>124.739990234375</v>
       </c>
       <c r="H5">
-        <v>155.03986328125</v>
+        <v>155.0400390625</v>
       </c>
       <c r="I5">
-        <v>-30.29995117187501</v>
+        <v>-30.300048828125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1093,13 +1093,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>166.7199609375</v>
+        <v>166.85986328125</v>
       </c>
       <c r="H2">
-        <v>126.219912109375</v>
+        <v>126.360107421875</v>
       </c>
       <c r="I2">
-        <v>40.50004882812499</v>
+        <v>40.499755859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1125,13 +1125,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>140.62005859375</v>
+        <v>140.76025390625</v>
       </c>
       <c r="H3">
-        <v>157.4601953125</v>
+        <v>157.60009765625</v>
       </c>
       <c r="I3">
-        <v>-16.84013671874999</v>
+        <v>-16.83984375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1157,13 +1157,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>135.139912109375</v>
+        <v>135.139892578125</v>
       </c>
       <c r="H4">
-        <v>134.6599609375</v>
+        <v>134.659912109375</v>
       </c>
       <c r="I4">
-        <v>0.4799511718750296</v>
+        <v>0.47998046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1189,13 +1189,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>125.4001953125</v>
+        <v>125.400146484375</v>
       </c>
       <c r="H5">
-        <v>149.54005859375</v>
+        <v>149.5400390625</v>
       </c>
       <c r="I5">
-        <v>-24.13986328125002</v>
+        <v>-24.139892578125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>166.869765625</v>
+        <v>166.86962890625</v>
       </c>
       <c r="H2">
-        <v>150.59990234375</v>
+        <v>150.60009765625</v>
       </c>
       <c r="I2">
-        <v>16.26986328125003</v>
+        <v>16.26953125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>161.4301953125</v>
+        <v>161.43017578125</v>
       </c>
       <c r="H3">
-        <v>146.939912109375</v>
+        <v>146.939697265625</v>
       </c>
       <c r="I3">
-        <v>14.49028320312502</v>
+        <v>14.490478515625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1327,13 +1327,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>156.67990234375</v>
+        <v>156.6796875</v>
       </c>
       <c r="H4">
-        <v>173.239765625</v>
+        <v>173.23974609375</v>
       </c>
       <c r="I4">
-        <v>-16.55986328125002</v>
+        <v>-16.56005859375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>140.859912109375</v>
+        <v>140.860107421875</v>
       </c>
       <c r="H5">
-        <v>155.0601953125</v>
+        <v>155.06005859375</v>
       </c>
       <c r="I5">
-        <v>-14.20028320312503</v>
+        <v>-14.199951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1433,13 +1433,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>159.04005859375</v>
+        <v>159.0400390625</v>
       </c>
       <c r="H2">
-        <v>130.590009765625</v>
+        <v>130.590087890625</v>
       </c>
       <c r="I2">
-        <v>28.45004882812503</v>
+        <v>28.449951171875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>152.529951171875</v>
+        <v>152.530029296875</v>
       </c>
       <c r="H3">
-        <v>155.73</v>
+        <v>155.72998046875</v>
       </c>
       <c r="I3">
-        <v>-3.200048828125034</v>
+        <v>-3.199951171875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1500,10 +1500,10 @@
         <v>137.760009765625</v>
       </c>
       <c r="H4">
-        <v>136.34005859375</v>
+        <v>136.33984375</v>
       </c>
       <c r="I4">
-        <v>1.419951171874999</v>
+        <v>1.420166015625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1529,13 +1529,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>133.03</v>
+        <v>133.02978515625</v>
       </c>
       <c r="H5">
         <v>159.699951171875</v>
       </c>
       <c r="I5">
-        <v>-26.669951171875</v>
+        <v>-26.670166015625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>146.4399609375</v>
+        <v>146.43994140625</v>
       </c>
       <c r="H2">
-        <v>135.36009765625</v>
+        <v>135.5</v>
       </c>
       <c r="I2">
-        <v>11.07986328125003</v>
+        <v>10.93994140625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>155.019765625</v>
+        <v>155.15966796875</v>
       </c>
       <c r="H3">
-        <v>142.08009765625</v>
+        <v>142.080078125</v>
       </c>
       <c r="I3">
-        <v>12.93966796874997</v>
+        <v>13.07958984375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1773,13 +1773,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>140.649951171875</v>
+        <v>140.650146484375</v>
       </c>
       <c r="H2">
-        <v>125.1399609375</v>
+        <v>125.14013671875</v>
       </c>
       <c r="I2">
-        <v>15.50999023437498</v>
+        <v>15.510009765625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>150.24005859375</v>
+        <v>150.240234375</v>
       </c>
       <c r="H3">
-        <v>142.1599609375</v>
+        <v>142.16015625</v>
       </c>
       <c r="I3">
-        <v>8.080097656250018</v>
+        <v>8.080078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>134.4399609375</v>
+        <v>134.43994140625</v>
       </c>
       <c r="H4">
-        <v>136.729951171875</v>
+        <v>136.729736328125</v>
       </c>
       <c r="I4">
-        <v>-2.289990234374983</v>
+        <v>-2.289794921875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1869,13 +1869,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>138.2399609375</v>
+        <v>138.23974609375</v>
       </c>
       <c r="H5">
-        <v>159.54005859375</v>
+        <v>159.5400390625</v>
       </c>
       <c r="I5">
-        <v>-21.30009765625002</v>
+        <v>-21.30029296875</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza datasets das parciais da rodada 3
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -62,27 +62,27 @@
     <t>JUV. KP</t>
   </si>
   <si>
+    <t>JV5 Tricolor Gaúcho</t>
+  </si>
+  <si>
     <t>SERGRILLO</t>
   </si>
   <si>
-    <t>JV5 Tricolor Gaúcho</t>
-  </si>
-  <si>
     <t>Grupo B</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>S.E.R. GRILLO</t>
   </si>
   <si>
+    <t>Máquina Laranjja</t>
+  </si>
+  <si>
     <t>Dom Camillo68</t>
   </si>
   <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
-    <t>Máquina Laranjja</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
@@ -92,12 +92,12 @@
     <t>cartola scheuer17</t>
   </si>
   <si>
+    <t>seralex</t>
+  </si>
+  <si>
     <t>dasdoresfc</t>
   </si>
   <si>
-    <t>seralex</t>
-  </si>
-  <si>
     <t>Grupo D</t>
   </si>
   <si>
@@ -116,58 +116,58 @@
     <t>Grupo E</t>
   </si>
   <si>
+    <t>KillerColorado</t>
+  </si>
+  <si>
+    <t>FÚRIA LEON</t>
+  </si>
+  <si>
+    <t>Fedato Futebol Clube</t>
+  </si>
+  <si>
     <t>Paulo Virgili FC</t>
   </si>
   <si>
-    <t>KillerColorado</t>
-  </si>
-  <si>
-    <t>Fedato Futebol Clube</t>
-  </si>
-  <si>
-    <t>FÚRIA LEON</t>
-  </si>
-  <si>
     <t>Grupo F</t>
   </si>
   <si>
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>AZURRA82</t>
+  </si>
+  <si>
     <t>DM Studio</t>
   </si>
   <si>
-    <t>AZURRA82</t>
-  </si>
-  <si>
     <t>Rolo Compressor ZN</t>
   </si>
   <si>
     <t>Grupo G</t>
   </si>
   <si>
+    <t>Grêmio imortal 37</t>
+  </si>
+  <si>
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
   </si>
   <si>
-    <t>Grêmio imortal 37</t>
-  </si>
-  <si>
     <t>A Lenda Super Vascão f.c</t>
   </si>
   <si>
     <t>Grupo H</t>
   </si>
   <si>
+    <t>Super Vasco f.c</t>
+  </si>
+  <si>
     <t>Gremiomaniasm</t>
   </si>
   <si>
     <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>Super Vasco f.c</t>
   </si>
   <si>
     <t>TEAM LOPES 99</t>
@@ -580,16 +580,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>159.56005859375</v>
+        <v>214.75005859375</v>
       </c>
       <c r="H2">
-        <v>91.030029296875</v>
+        <v>153.830029296875</v>
       </c>
       <c r="I2">
-        <v>68.530029296875</v>
+        <v>60.92002929687499</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -603,10 +603,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>140.18017578125</v>
+        <v>198.55017578125</v>
       </c>
       <c r="H3">
-        <v>139.0400390625</v>
+        <v>156.5400390625</v>
       </c>
       <c r="I3">
-        <v>1.14013671875</v>
+        <v>42.01013671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -644,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>85.429931640625</v>
+        <v>182.840283203125</v>
       </c>
       <c r="H4">
-        <v>140.560302734375</v>
+        <v>189.770078125</v>
       </c>
       <c r="I4">
-        <v>-55.13037109375</v>
+        <v>-6.929794921874986</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -667,10 +667,10 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -679,13 +679,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>120.040283203125</v>
+        <v>102.929931640625</v>
       </c>
       <c r="H5">
-        <v>134.580078125</v>
+        <v>198.930302734375</v>
       </c>
       <c r="I5">
-        <v>-14.539794921875</v>
+        <v>-96.00037109375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -750,16 +750,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>164.31005859375</v>
+        <v>199.009990234375</v>
       </c>
       <c r="H2">
-        <v>114.340087890625</v>
+        <v>171.78017578125</v>
       </c>
       <c r="I2">
-        <v>49.969970703125</v>
+        <v>27.22981445312499</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -773,10 +773,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -785,13 +785,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>137.2802734375</v>
+        <v>185.91005859375</v>
       </c>
       <c r="H3">
-        <v>127.310302734375</v>
+        <v>183.610087890625</v>
       </c>
       <c r="I3">
-        <v>9.969970703125</v>
+        <v>2.299970703125013</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -814,16 +814,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>129.739990234375</v>
+        <v>197.609990234375</v>
       </c>
       <c r="H4">
-        <v>150.18017578125</v>
+        <v>225.13974609375</v>
       </c>
       <c r="I4">
-        <v>-20.440185546875</v>
+        <v>-27.529755859375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,10 +837,10 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -849,13 +849,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>127.239990234375</v>
+        <v>195.6802734375</v>
       </c>
       <c r="H5">
-        <v>166.73974609375</v>
+        <v>197.680302734375</v>
       </c>
       <c r="I5">
-        <v>-39.499755859375</v>
+        <v>-2.000029296874999</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>167.83984375</v>
+        <v>222.80984375</v>
       </c>
       <c r="H2">
-        <v>126.7099609375</v>
+        <v>184.1799609375</v>
       </c>
       <c r="I2">
-        <v>41.1298828125</v>
+        <v>38.6298828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -943,10 +943,10 @@
         <v>22</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -955,13 +955,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>143.740234375</v>
+        <v>188.910234375</v>
       </c>
       <c r="H3">
-        <v>138.64013671875</v>
+        <v>181.10013671875</v>
       </c>
       <c r="I3">
-        <v>5.10009765625</v>
+        <v>7.810097656250008</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -984,16 +984,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>138.009765625</v>
+        <v>182.209990234375</v>
       </c>
       <c r="H4">
-        <v>153.939697265625</v>
+        <v>210.0100390625</v>
       </c>
       <c r="I4">
-        <v>-15.929931640625</v>
+        <v>-27.800048828125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1007,10 +1007,10 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1019,13 +1019,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>124.739990234375</v>
+        <v>180.469765625</v>
       </c>
       <c r="H5">
-        <v>155.0400390625</v>
+        <v>199.109697265625</v>
       </c>
       <c r="I5">
-        <v>-30.300048828125</v>
+        <v>-18.63993164062501</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1081,10 +1081,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1093,13 +1093,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>166.85986328125</v>
+        <v>214.42986328125</v>
       </c>
       <c r="H2">
-        <v>126.360107421875</v>
+        <v>166.530107421875</v>
       </c>
       <c r="I2">
-        <v>40.499755859375</v>
+        <v>47.89975585937498</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,22 +1113,22 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>140.76025390625</v>
+        <v>178.83025390625</v>
       </c>
       <c r="H3">
-        <v>157.60009765625</v>
+        <v>195.67009765625</v>
       </c>
       <c r="I3">
         <v>-16.83984375</v>
@@ -1145,22 +1145,22 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>135.139892578125</v>
+        <v>173.209892578125</v>
       </c>
       <c r="H4">
-        <v>134.659912109375</v>
+        <v>172.729912109375</v>
       </c>
       <c r="I4">
         <v>0.47998046875</v>
@@ -1186,16 +1186,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>125.400146484375</v>
+        <v>165.570146484375</v>
       </c>
       <c r="H5">
-        <v>149.5400390625</v>
+        <v>197.1100390625</v>
       </c>
       <c r="I5">
-        <v>-24.139892578125</v>
+        <v>-31.53989257812498</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1251,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>166.86962890625</v>
+        <v>218.60017578125</v>
       </c>
       <c r="H2">
-        <v>150.60009765625</v>
+        <v>176.139697265625</v>
       </c>
       <c r="I2">
-        <v>16.26953125</v>
+        <v>42.46047851562503</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1283,10 +1283,10 @@
         <v>32</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>161.43017578125</v>
+        <v>200.730107421875</v>
       </c>
       <c r="H3">
-        <v>146.939697265625</v>
+        <v>195.66005859375</v>
       </c>
       <c r="I3">
-        <v>14.490478515625</v>
+        <v>5.07004882812501</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1324,16 +1324,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>156.6796875</v>
+        <v>197.2796875</v>
       </c>
       <c r="H4">
-        <v>173.23974609375</v>
+        <v>233.10974609375</v>
       </c>
       <c r="I4">
-        <v>-16.56005859375</v>
+        <v>-35.83005859375001</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>140.860107421875</v>
+        <v>196.06962890625</v>
       </c>
       <c r="H5">
-        <v>155.06005859375</v>
+        <v>207.77009765625</v>
       </c>
       <c r="I5">
-        <v>-14.199951171875</v>
+        <v>-11.70046875000003</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1430,16 +1430,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>159.0400390625</v>
+        <v>212.8100390625</v>
       </c>
       <c r="H2">
-        <v>130.590087890625</v>
+        <v>184.860087890625</v>
       </c>
       <c r="I2">
-        <v>28.449951171875</v>
+        <v>27.949951171875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1453,10 +1453,10 @@
         <v>37</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1465,13 +1465,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>152.530029296875</v>
+        <v>205.030009765625</v>
       </c>
       <c r="H3">
-        <v>155.72998046875</v>
+        <v>174.60984375</v>
       </c>
       <c r="I3">
-        <v>-3.199951171875</v>
+        <v>30.42016601562497</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1494,16 +1494,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>137.760009765625</v>
+        <v>190.800029296875</v>
       </c>
       <c r="H4">
-        <v>136.33984375</v>
+        <v>222.99998046875</v>
       </c>
       <c r="I4">
-        <v>1.420166015625</v>
+        <v>-32.19995117187497</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1517,10 +1517,10 @@
         <v>39</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1529,13 +1529,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>133.02978515625</v>
+        <v>187.29978515625</v>
       </c>
       <c r="H5">
-        <v>159.699951171875</v>
+        <v>213.469951171875</v>
       </c>
       <c r="I5">
-        <v>-26.670166015625</v>
+        <v>-26.170166015625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1600,16 +1600,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>146.43994140625</v>
+        <v>181.97009765625</v>
       </c>
       <c r="H2">
-        <v>135.5</v>
+        <v>191.259765625</v>
       </c>
       <c r="I2">
-        <v>10.93994140625</v>
+        <v>-9.289667968749995</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1623,10 +1623,10 @@
         <v>42</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>155.15966796875</v>
+        <v>181.93994140625</v>
       </c>
       <c r="H3">
-        <v>142.080078125</v>
+        <v>175.37</v>
       </c>
       <c r="I3">
-        <v>13.07958984375</v>
+        <v>6.569941406249995</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1664,16 +1664,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>142.10009765625</v>
+        <v>195.72966796875</v>
       </c>
       <c r="H4">
-        <v>155.759765625</v>
+        <v>192.850078125</v>
       </c>
       <c r="I4">
-        <v>-13.65966796875</v>
+        <v>2.879589843749983</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1687,10 +1687,10 @@
         <v>44</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1699,13 +1699,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>136.10009765625</v>
+        <v>186.87009765625</v>
       </c>
       <c r="H5">
-        <v>146.4599609375</v>
+        <v>187.0299609375</v>
       </c>
       <c r="I5">
-        <v>-10.35986328125</v>
+        <v>-0.1598632812499829</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1770,16 +1770,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>140.650146484375</v>
+        <v>192.90994140625</v>
       </c>
       <c r="H2">
-        <v>125.14013671875</v>
+        <v>181.899736328125</v>
       </c>
       <c r="I2">
-        <v>15.510009765625</v>
+        <v>11.01020507812498</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1793,10 +1793,10 @@
         <v>47</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1805,13 +1805,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>150.240234375</v>
+        <v>168.550146484375</v>
       </c>
       <c r="H3">
-        <v>142.16015625</v>
+        <v>170.91013671875</v>
       </c>
       <c r="I3">
-        <v>8.080078125</v>
+        <v>-2.359990234375005</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1834,16 +1834,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>134.43994140625</v>
+        <v>195.410234375</v>
       </c>
       <c r="H4">
-        <v>136.729736328125</v>
+        <v>200.63015625</v>
       </c>
       <c r="I4">
-        <v>-2.289794921875</v>
+        <v>-5.219921874999983</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1857,10 +1857,10 @@
         <v>49</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1869,13 +1869,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>138.23974609375</v>
+        <v>184.00974609375</v>
       </c>
       <c r="H5">
-        <v>159.5400390625</v>
+        <v>187.4400390625</v>
       </c>
       <c r="I5">
-        <v>-21.30029296875</v>
+        <v>-3.430292968749995</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza datasets com nova parcial
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -71,18 +71,18 @@
     <t>Grupo B</t>
   </si>
   <si>
+    <t>S.E.R. GRILLO</t>
+  </si>
+  <si>
+    <t>Dom Camillo68</t>
+  </si>
+  <si>
     <t>LISI GREMISTA</t>
   </si>
   <si>
-    <t>S.E.R. GRILLO</t>
-  </si>
-  <si>
     <t>Máquina Laranjja</t>
   </si>
   <si>
-    <t>Dom Camillo68</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
@@ -92,12 +92,12 @@
     <t>cartola scheuer17</t>
   </si>
   <si>
+    <t>dasdoresfc</t>
+  </si>
+  <si>
     <t>seralex</t>
   </si>
   <si>
-    <t>dasdoresfc</t>
-  </si>
-  <si>
     <t>Grupo D</t>
   </si>
   <si>
@@ -119,55 +119,55 @@
     <t>KillerColorado</t>
   </si>
   <si>
+    <t>Fedato Futebol Clube</t>
+  </si>
+  <si>
+    <t>Paulo Virgili FC</t>
+  </si>
+  <si>
     <t>FÚRIA LEON</t>
   </si>
   <si>
-    <t>Fedato Futebol Clube</t>
-  </si>
-  <si>
-    <t>Paulo Virgili FC</t>
-  </si>
-  <si>
     <t>Grupo F</t>
   </si>
   <si>
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>DM Studio</t>
+  </si>
+  <si>
+    <t>Rolo Compressor ZN</t>
+  </si>
+  <si>
     <t>AZURRA82</t>
   </si>
   <si>
-    <t>DM Studio</t>
-  </si>
-  <si>
-    <t>Rolo Compressor ZN</t>
-  </si>
-  <si>
     <t>Grupo G</t>
   </si>
   <si>
+    <t>Tabajara de Inhaua PB1</t>
+  </si>
+  <si>
+    <t>TORRESMO COM PINGA PRO26.1</t>
+  </si>
+  <si>
     <t>Grêmio imortal 37</t>
   </si>
   <si>
-    <t>Tabajara de Inhaua PB1</t>
-  </si>
-  <si>
-    <t>TORRESMO COM PINGA PRO26.1</t>
-  </si>
-  <si>
     <t>A Lenda Super Vascão f.c</t>
   </si>
   <si>
     <t>Grupo H</t>
   </si>
   <si>
+    <t>Texas Club 2026</t>
+  </si>
+  <si>
+    <t>Gremiomaniasm</t>
+  </si>
+  <si>
     <t>Super Vasco f.c</t>
-  </si>
-  <si>
-    <t>Gremiomaniasm</t>
-  </si>
-  <si>
-    <t>Texas Club 2026</t>
   </si>
   <si>
     <t>TEAM LOPES 99</t>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>214.75005859375</v>
+        <v>232.80005859375</v>
       </c>
       <c r="H2">
-        <v>153.830029296875</v>
+        <v>188.430029296875</v>
       </c>
       <c r="I2">
-        <v>60.92002929687499</v>
+        <v>44.370029296875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -615,13 +615,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>198.55017578125</v>
+        <v>207.14017578125</v>
       </c>
       <c r="H3">
-        <v>156.5400390625</v>
+        <v>192.1900390625</v>
       </c>
       <c r="I3">
-        <v>42.01013671875</v>
+        <v>14.95013671874997</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -647,13 +647,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>182.840283203125</v>
+        <v>217.440283203125</v>
       </c>
       <c r="H4">
-        <v>189.770078125</v>
+        <v>207.820078125</v>
       </c>
       <c r="I4">
-        <v>-6.929794921874986</v>
+        <v>9.620205078124997</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>102.929931640625</v>
+        <v>138.579931640625</v>
       </c>
       <c r="H5">
-        <v>198.930302734375</v>
+        <v>207.520302734375</v>
       </c>
       <c r="I5">
-        <v>-96.00037109375</v>
+        <v>-68.94037109374997</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>199.009990234375</v>
+        <v>242.57005859375</v>
       </c>
       <c r="H2">
-        <v>171.78017578125</v>
+        <v>212.100087890625</v>
       </c>
       <c r="I2">
-        <v>27.22981445312499</v>
+        <v>30.469970703125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -785,13 +785,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>185.91005859375</v>
+        <v>235.9302734375</v>
       </c>
       <c r="H3">
-        <v>183.610087890625</v>
+        <v>207.770302734375</v>
       </c>
       <c r="I3">
-        <v>2.299970703125013</v>
+        <v>28.15997070312503</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -805,25 +805,25 @@
         <v>18</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>197.609990234375</v>
+        <v>227.499990234375</v>
       </c>
       <c r="H4">
-        <v>225.13974609375</v>
+        <v>228.44017578125</v>
       </c>
       <c r="I4">
-        <v>-27.529755859375</v>
+        <v>-0.940185546875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,25 +837,25 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>195.6802734375</v>
+        <v>207.699990234375</v>
       </c>
       <c r="H5">
-        <v>197.680302734375</v>
+        <v>265.38974609375</v>
       </c>
       <c r="I5">
-        <v>-2.000029296874999</v>
+        <v>-57.689755859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -911,25 +911,25 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>222.80984375</v>
+        <v>261.29984375</v>
       </c>
       <c r="H2">
-        <v>184.1799609375</v>
+        <v>215.4699609375</v>
       </c>
       <c r="I2">
-        <v>38.6298828125</v>
+        <v>45.82988281249999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -955,13 +955,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>188.910234375</v>
+        <v>249.500234375</v>
       </c>
       <c r="H3">
-        <v>181.10013671875</v>
+        <v>219.35013671875</v>
       </c>
       <c r="I3">
-        <v>7.810097656250008</v>
+        <v>30.15009765625001</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,13 +987,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>182.209990234375</v>
+        <v>218.719765625</v>
       </c>
       <c r="H4">
-        <v>210.0100390625</v>
+        <v>259.699697265625</v>
       </c>
       <c r="I4">
-        <v>-27.800048828125</v>
+        <v>-40.97993164062501</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1007,25 +1007,25 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>180.469765625</v>
+        <v>213.499990234375</v>
       </c>
       <c r="H5">
-        <v>199.109697265625</v>
+        <v>248.5000390625</v>
       </c>
       <c r="I5">
-        <v>-18.63993164062501</v>
+        <v>-35.00004882812499</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1081,25 +1081,25 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>214.42986328125</v>
+        <v>248.61986328125</v>
       </c>
       <c r="H2">
-        <v>166.530107421875</v>
+        <v>212.520107421875</v>
       </c>
       <c r="I2">
-        <v>47.89975585937498</v>
+        <v>36.09975585937499</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,25 +1113,25 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>178.83025390625</v>
+        <v>219.82025390625</v>
       </c>
       <c r="H3">
-        <v>195.67009765625</v>
+        <v>236.06009765625</v>
       </c>
       <c r="I3">
-        <v>-16.83984375</v>
+        <v>-16.23984374999998</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1145,25 +1145,25 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>173.209892578125</v>
+        <v>213.599892578125</v>
       </c>
       <c r="H4">
-        <v>172.729912109375</v>
+        <v>213.719912109375</v>
       </c>
       <c r="I4">
-        <v>0.47998046875</v>
+        <v>-0.1200195312500227</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1177,25 +1177,25 @@
         <v>29</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>165.570146484375</v>
+        <v>211.560146484375</v>
       </c>
       <c r="H5">
-        <v>197.1100390625</v>
+        <v>231.3000390625</v>
       </c>
       <c r="I5">
-        <v>-31.53989257812498</v>
+        <v>-19.73989257812499</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>218.60017578125</v>
+        <v>244.89017578125</v>
       </c>
       <c r="H2">
-        <v>176.139697265625</v>
+        <v>228.189697265625</v>
       </c>
       <c r="I2">
-        <v>42.46047851562503</v>
+        <v>16.70047851562498</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>200.730107421875</v>
+        <v>235.0796875</v>
       </c>
       <c r="H3">
-        <v>195.66005859375</v>
+        <v>247.99974609375</v>
       </c>
       <c r="I3">
-        <v>5.07004882812501</v>
+        <v>-12.92005859374999</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1327,13 +1327,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>197.2796875</v>
+        <v>248.11962890625</v>
       </c>
       <c r="H4">
-        <v>233.10974609375</v>
+        <v>234.06009765625</v>
       </c>
       <c r="I4">
-        <v>-35.83005859375001</v>
+        <v>14.05953125000002</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>196.06962890625</v>
+        <v>215.620107421875</v>
       </c>
       <c r="H5">
-        <v>207.77009765625</v>
+        <v>233.46005859375</v>
       </c>
       <c r="I5">
-        <v>-11.70046875000003</v>
+        <v>-17.83995117187501</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>212.8100390625</v>
+        <v>246.5000390625</v>
       </c>
       <c r="H2">
-        <v>184.860087890625</v>
+        <v>223.550087890625</v>
       </c>
       <c r="I2">
-        <v>27.949951171875</v>
+        <v>22.949951171875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>205.030009765625</v>
+        <v>232.290029296875</v>
       </c>
       <c r="H3">
-        <v>174.60984375</v>
+        <v>226.78998046875</v>
       </c>
       <c r="I3">
-        <v>30.42016601562497</v>
+        <v>5.500048828124989</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1497,13 +1497,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>190.800029296875</v>
+        <v>225.98978515625</v>
       </c>
       <c r="H4">
-        <v>222.99998046875</v>
+        <v>247.159951171875</v>
       </c>
       <c r="I4">
-        <v>-32.19995117187497</v>
+        <v>-21.170166015625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1529,13 +1529,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>187.29978515625</v>
+        <v>208.820009765625</v>
       </c>
       <c r="H5">
-        <v>213.469951171875</v>
+        <v>216.09984375</v>
       </c>
       <c r="I5">
-        <v>-26.170166015625</v>
+        <v>-7.279833984374989</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,25 +1591,25 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>181.97009765625</v>
+        <v>233.83994140625</v>
       </c>
       <c r="H2">
-        <v>191.259765625</v>
+        <v>214.36</v>
       </c>
       <c r="I2">
-        <v>-9.289667968749995</v>
+        <v>19.47994140624999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>181.93994140625</v>
+        <v>235.71966796875</v>
       </c>
       <c r="H3">
-        <v>175.37</v>
+        <v>214.240078125</v>
       </c>
       <c r="I3">
-        <v>6.569941406249995</v>
+        <v>21.47958984375001</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1667,13 +1667,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>195.72966796875</v>
+        <v>220.96009765625</v>
       </c>
       <c r="H4">
-        <v>192.850078125</v>
+        <v>243.159765625</v>
       </c>
       <c r="I4">
-        <v>2.879589843749983</v>
+        <v>-22.19966796874999</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1687,25 +1687,25 @@
         <v>44</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>186.87009765625</v>
+        <v>208.26009765625</v>
       </c>
       <c r="H5">
-        <v>187.0299609375</v>
+        <v>227.0199609375</v>
       </c>
       <c r="I5">
-        <v>-0.1598632812499829</v>
+        <v>-18.75986328125001</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1773,13 +1773,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>192.90994140625</v>
+        <v>256.000234375</v>
       </c>
       <c r="H2">
-        <v>181.899736328125</v>
+        <v>240.72015625</v>
       </c>
       <c r="I2">
-        <v>11.01020507812498</v>
+        <v>15.28007812499999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>168.550146484375</v>
+        <v>211.450146484375</v>
       </c>
       <c r="H3">
-        <v>170.91013671875</v>
+        <v>211.80013671875</v>
       </c>
       <c r="I3">
-        <v>-2.359990234375005</v>
+        <v>-0.3499902343749852</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>195.410234375</v>
+        <v>232.99994140625</v>
       </c>
       <c r="H4">
-        <v>200.63015625</v>
+        <v>242.489736328125</v>
       </c>
       <c r="I4">
-        <v>-5.219921874999983</v>
+        <v>-9.489794921874989</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1869,13 +1869,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>184.00974609375</v>
+        <v>224.89974609375</v>
       </c>
       <c r="H5">
-        <v>187.4400390625</v>
+        <v>230.3400390625</v>
       </c>
       <c r="I5">
-        <v>-3.430292968749995</v>
+        <v>-5.440292968750015</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Fecha datasets da rodada 3
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>232.80005859375</v>
+        <v>232.30029296875</v>
       </c>
       <c r="H2">
-        <v>188.430029296875</v>
+        <v>188.429931640625</v>
       </c>
       <c r="I2">
-        <v>44.370029296875</v>
+        <v>43.870361328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -615,13 +615,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>207.14017578125</v>
+        <v>207.93994140625</v>
       </c>
       <c r="H3">
-        <v>192.1900390625</v>
+        <v>193.39013671875</v>
       </c>
       <c r="I3">
-        <v>14.95013671874997</v>
+        <v>14.5498046875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -647,13 +647,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>217.440283203125</v>
+        <v>217.440185546875</v>
       </c>
       <c r="H4">
-        <v>207.820078125</v>
+        <v>207.3203125</v>
       </c>
       <c r="I4">
-        <v>9.620205078124997</v>
+        <v>10.119873046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>138.579931640625</v>
+        <v>139.780029296875</v>
       </c>
       <c r="H5">
-        <v>207.520302734375</v>
+        <v>208.320068359375</v>
       </c>
       <c r="I5">
-        <v>-68.94037109374997</v>
+        <v>-68.5400390625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>242.57005859375</v>
+        <v>243.25</v>
       </c>
       <c r="H2">
-        <v>212.100087890625</v>
+        <v>212.099853515625</v>
       </c>
       <c r="I2">
-        <v>30.469970703125</v>
+        <v>31.150146484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -785,13 +785,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>235.9302734375</v>
+        <v>235.93017578125</v>
       </c>
       <c r="H3">
-        <v>207.770302734375</v>
+        <v>208.570068359375</v>
       </c>
       <c r="I3">
-        <v>28.15997070312503</v>
+        <v>27.360107421875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -817,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>227.499990234375</v>
+        <v>227.499755859375</v>
       </c>
       <c r="H4">
-        <v>228.44017578125</v>
+        <v>229.1201171875</v>
       </c>
       <c r="I4">
-        <v>-0.940185546875</v>
+        <v>-1.620361328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -849,13 +849,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>207.699990234375</v>
+        <v>208.499755859375</v>
       </c>
       <c r="H5">
-        <v>265.38974609375</v>
+        <v>265.3896484375</v>
       </c>
       <c r="I5">
-        <v>-57.689755859375</v>
+        <v>-56.889892578125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>261.29984375</v>
+        <v>262.099609375</v>
       </c>
       <c r="H2">
-        <v>215.4699609375</v>
+        <v>215.4697265625</v>
       </c>
       <c r="I2">
-        <v>45.82988281249999</v>
+        <v>46.6298828125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -955,13 +955,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>249.500234375</v>
+        <v>249.5</v>
       </c>
       <c r="H3">
-        <v>219.35013671875</v>
+        <v>218.93994140625</v>
       </c>
       <c r="I3">
-        <v>30.15009765625001</v>
+        <v>30.56005859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,13 +987,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>218.719765625</v>
+        <v>218.3095703125</v>
       </c>
       <c r="H4">
-        <v>259.699697265625</v>
+        <v>259.699462890625</v>
       </c>
       <c r="I4">
-        <v>-40.97993164062501</v>
+        <v>-41.389892578125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1019,13 +1019,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>213.499990234375</v>
+        <v>213.499755859375</v>
       </c>
       <c r="H5">
-        <v>248.5000390625</v>
+        <v>249.2998046875</v>
       </c>
       <c r="I5">
-        <v>-35.00004882812499</v>
+        <v>-35.800048828125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1093,13 +1093,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>248.61986328125</v>
+        <v>248.61962890625</v>
       </c>
       <c r="H2">
-        <v>212.520107421875</v>
+        <v>212.520263671875</v>
       </c>
       <c r="I2">
-        <v>36.09975585937499</v>
+        <v>36.099365234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1125,13 +1125,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>219.82025390625</v>
+        <v>220.6201171875</v>
       </c>
       <c r="H3">
-        <v>236.06009765625</v>
+        <v>236.85986328125</v>
       </c>
       <c r="I3">
-        <v>-16.23984374999998</v>
+        <v>-16.23974609375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1157,13 +1157,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>213.599892578125</v>
+        <v>214.399658203125</v>
       </c>
       <c r="H4">
-        <v>213.719912109375</v>
+        <v>214.519775390625</v>
       </c>
       <c r="I4">
-        <v>-0.1200195312500227</v>
+        <v>-0.1201171875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1189,13 +1189,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>211.560146484375</v>
+        <v>211.560302734375</v>
       </c>
       <c r="H5">
-        <v>231.3000390625</v>
+        <v>231.2998046875</v>
       </c>
       <c r="I5">
-        <v>-19.73989257812499</v>
+        <v>-19.739501953125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>244.89017578125</v>
+        <v>245.68994140625</v>
       </c>
       <c r="H2">
         <v>228.189697265625</v>
       </c>
       <c r="I2">
-        <v>16.70047851562498</v>
+        <v>17.500244140625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>235.0796875</v>
+        <v>235.07958984375</v>
       </c>
       <c r="H3">
-        <v>247.99974609375</v>
+        <v>248.7998046875</v>
       </c>
       <c r="I3">
-        <v>-12.92005859374999</v>
+        <v>-13.72021484375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1330,10 +1330,10 @@
         <v>248.11962890625</v>
       </c>
       <c r="H4">
-        <v>234.06009765625</v>
+        <v>234.85986328125</v>
       </c>
       <c r="I4">
-        <v>14.05953125000002</v>
+        <v>13.259765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>215.620107421875</v>
+        <v>216.420166015625</v>
       </c>
       <c r="H5">
-        <v>233.46005859375</v>
+        <v>233.4599609375</v>
       </c>
       <c r="I5">
-        <v>-17.83995117187501</v>
+        <v>-17.039794921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>246.5000390625</v>
+        <v>246.5</v>
       </c>
       <c r="H2">
-        <v>223.550087890625</v>
+        <v>224.349853515625</v>
       </c>
       <c r="I2">
-        <v>22.949951171875</v>
+        <v>22.150146484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>232.290029296875</v>
+        <v>233.090087890625</v>
       </c>
       <c r="H3">
-        <v>226.78998046875</v>
+        <v>227.58984375</v>
       </c>
       <c r="I3">
-        <v>5.500048828124989</v>
+        <v>5.500244140625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1497,13 +1497,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>225.98978515625</v>
+        <v>226.78955078125</v>
       </c>
       <c r="H4">
-        <v>247.159951171875</v>
+        <v>247.159912109375</v>
       </c>
       <c r="I4">
-        <v>-21.170166015625</v>
+        <v>-20.370361328125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1529,13 +1529,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>208.820009765625</v>
+        <v>209.619873046875</v>
       </c>
       <c r="H5">
-        <v>216.09984375</v>
+        <v>216.89990234375</v>
       </c>
       <c r="I5">
-        <v>-7.279833984374989</v>
+        <v>-7.280029296875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>233.83994140625</v>
+        <v>233.83984375</v>
       </c>
       <c r="H2">
-        <v>214.36</v>
+        <v>214.35986328125</v>
       </c>
       <c r="I2">
-        <v>19.47994140624999</v>
+        <v>19.47998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>235.71966796875</v>
+        <v>236.51953125</v>
       </c>
       <c r="H3">
-        <v>214.240078125</v>
+        <v>215.0400390625</v>
       </c>
       <c r="I3">
-        <v>21.47958984375001</v>
+        <v>21.4794921875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1667,13 +1667,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>220.96009765625</v>
+        <v>220.9599609375</v>
       </c>
       <c r="H4">
-        <v>243.159765625</v>
+        <v>243.15966796875</v>
       </c>
       <c r="I4">
-        <v>-22.19966796874999</v>
+        <v>-22.19970703125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1699,13 +1699,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>208.26009765625</v>
+        <v>209.06005859375</v>
       </c>
       <c r="H5">
-        <v>227.0199609375</v>
+        <v>227.81982421875</v>
       </c>
       <c r="I5">
-        <v>-18.75986328125001</v>
+        <v>-18.759765625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1773,13 +1773,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>256.000234375</v>
+        <v>256</v>
       </c>
       <c r="H2">
-        <v>240.72015625</v>
+        <v>241.52001953125</v>
       </c>
       <c r="I2">
-        <v>15.28007812499999</v>
+        <v>14.47998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>211.450146484375</v>
+        <v>211.449951171875</v>
       </c>
       <c r="H3">
-        <v>211.80013671875</v>
+        <v>211.80029296875</v>
       </c>
       <c r="I3">
-        <v>-0.3499902343749852</v>
+        <v>-0.350341796875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>232.99994140625</v>
+        <v>233.7998046875</v>
       </c>
       <c r="H4">
-        <v>242.489736328125</v>
+        <v>242.489501953125</v>
       </c>
       <c r="I4">
-        <v>-9.489794921874989</v>
+        <v>-8.689697265625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1869,13 +1869,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>224.89974609375</v>
+        <v>224.89990234375</v>
       </c>
       <c r="H5">
-        <v>230.3400390625</v>
+        <v>230.33984375</v>
       </c>
       <c r="I5">
-        <v>-5.440292968750015</v>
+        <v>-5.43994140625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza parciais da rodada 4
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -59,27 +59,27 @@
     <t>Tatols Beants F.C</t>
   </si>
   <si>
+    <t>JV5 Tricolor Gaúcho</t>
+  </si>
+  <si>
     <t>JUV. KP</t>
   </si>
   <si>
-    <t>JV5 Tricolor Gaúcho</t>
-  </si>
-  <si>
     <t>SERGRILLO</t>
   </si>
   <si>
     <t>Grupo B</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
+    <t>Dom Camillo68</t>
+  </si>
+  <si>
     <t>S.E.R. GRILLO</t>
   </si>
   <si>
-    <t>Dom Camillo68</t>
-  </si>
-  <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
     <t>Máquina Laranjja</t>
   </si>
   <si>
@@ -101,45 +101,45 @@
     <t>Grupo D</t>
   </si>
   <si>
+    <t>A Lenda Super Vasco F.c</t>
+  </si>
+  <si>
+    <t>FBC Colorado</t>
+  </si>
+  <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
-    <t>A Lenda Super Vasco F.c</t>
-  </si>
-  <si>
-    <t>FBC Colorado</t>
-  </si>
-  <si>
     <t>Grêmio imortal 36</t>
   </si>
   <si>
     <t>Grupo E</t>
   </si>
   <si>
+    <t>Fedato Futebol Clube</t>
+  </si>
+  <si>
     <t>KillerColorado</t>
   </si>
   <si>
-    <t>Fedato Futebol Clube</t>
+    <t>FÚRIA LEON</t>
   </si>
   <si>
     <t>Paulo Virgili FC</t>
   </si>
   <si>
-    <t>FÚRIA LEON</t>
-  </si>
-  <si>
     <t>Grupo F</t>
   </si>
   <si>
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>Rolo Compressor ZN</t>
+  </si>
+  <si>
     <t>DM Studio</t>
   </si>
   <si>
-    <t>Rolo Compressor ZN</t>
-  </si>
-  <si>
     <t>AZURRA82</t>
   </si>
   <si>
@@ -149,28 +149,28 @@
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
+    <t>Grêmio imortal 37</t>
+  </si>
+  <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
   </si>
   <si>
-    <t>Grêmio imortal 37</t>
-  </si>
-  <si>
     <t>A Lenda Super Vascão f.c</t>
   </si>
   <si>
     <t>Grupo H</t>
   </si>
   <si>
+    <t>Gremiomaniasm</t>
+  </si>
+  <si>
     <t>Texas Club 2026</t>
   </si>
   <si>
-    <t>Gremiomaniasm</t>
+    <t>TEAM LOPES 99</t>
   </si>
   <si>
     <t>Super Vasco f.c</t>
-  </si>
-  <si>
-    <t>TEAM LOPES 99</t>
   </si>
 </sst>
 </file>
@@ -571,10 +571,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>232.30029296875</v>
+        <v>281.19029296875</v>
       </c>
       <c r="H2">
-        <v>188.429931640625</v>
+        <v>210.079931640625</v>
       </c>
       <c r="I2">
-        <v>43.870361328125</v>
+        <v>71.11036132812498</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>207.93994140625</v>
+        <v>282.990185546875</v>
       </c>
       <c r="H3">
-        <v>193.39013671875</v>
+        <v>243.0203125</v>
       </c>
       <c r="I3">
-        <v>14.5498046875</v>
+        <v>39.96987304687502</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -635,10 +635,10 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -647,13 +647,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>217.440185546875</v>
+        <v>243.63994140625</v>
       </c>
       <c r="H4">
-        <v>207.3203125</v>
+        <v>258.94013671875</v>
       </c>
       <c r="I4">
-        <v>10.119873046875</v>
+        <v>-15.30019531250002</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -676,16 +676,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>139.780029296875</v>
+        <v>161.430029296875</v>
       </c>
       <c r="H5">
-        <v>208.320068359375</v>
+        <v>257.210068359375</v>
       </c>
       <c r="I5">
-        <v>-68.5400390625</v>
+        <v>-95.78003906249998</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>243.25</v>
+        <v>293.049755859375</v>
       </c>
       <c r="H2">
-        <v>212.099853515625</v>
+        <v>277.1001171875</v>
       </c>
       <c r="I2">
-        <v>31.150146484375</v>
+        <v>15.94963867187499</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -773,10 +773,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -785,13 +785,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>235.93017578125</v>
+        <v>278.23017578125</v>
       </c>
       <c r="H3">
-        <v>208.570068359375</v>
+        <v>240.350068359375</v>
       </c>
       <c r="I3">
-        <v>27.360107421875</v>
+        <v>37.88010742187501</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -814,16 +814,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>227.499755859375</v>
+        <v>275.03</v>
       </c>
       <c r="H4">
-        <v>229.1201171875</v>
+        <v>254.399853515625</v>
       </c>
       <c r="I4">
-        <v>-1.620361328125</v>
+        <v>20.63014648437496</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -846,16 +846,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>208.499755859375</v>
+        <v>256.479755859375</v>
       </c>
       <c r="H5">
-        <v>265.3896484375</v>
+        <v>330.9396484375</v>
       </c>
       <c r="I5">
-        <v>-56.889892578125</v>
+        <v>-74.45989257812499</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -920,16 +920,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>262.099609375</v>
+        <v>308.649609375</v>
       </c>
       <c r="H2">
-        <v>215.4697265625</v>
+        <v>271.8697265625</v>
       </c>
       <c r="I2">
-        <v>46.6298828125</v>
+        <v>36.77988281250003</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>249.5</v>
+        <v>293.3</v>
       </c>
       <c r="H3">
-        <v>218.93994140625</v>
+        <v>277.13994140625</v>
       </c>
       <c r="I3">
-        <v>30.56005859375</v>
+        <v>16.16005859375002</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -975,10 +975,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -987,13 +987,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>218.3095703125</v>
+        <v>274.7095703125</v>
       </c>
       <c r="H4">
-        <v>259.699462890625</v>
+        <v>306.249462890625</v>
       </c>
       <c r="I4">
-        <v>-41.389892578125</v>
+        <v>-31.53989257812503</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1007,10 +1007,10 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1019,13 +1019,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>213.499755859375</v>
+        <v>271.699755859375</v>
       </c>
       <c r="H5">
-        <v>249.2998046875</v>
+        <v>293.0998046875</v>
       </c>
       <c r="I5">
-        <v>-35.800048828125</v>
+        <v>-21.40004882812502</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1081,10 +1081,10 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1093,13 +1093,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>248.61962890625</v>
+        <v>253.3501171875</v>
       </c>
       <c r="H2">
-        <v>212.520263671875</v>
+        <v>262.15986328125</v>
       </c>
       <c r="I2">
-        <v>36.099365234375</v>
+        <v>-8.809746093750022</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1122,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>220.6201171875</v>
+        <v>273.929658203125</v>
       </c>
       <c r="H3">
-        <v>236.85986328125</v>
+        <v>261.969775390625</v>
       </c>
       <c r="I3">
-        <v>-16.23974609375</v>
+        <v>11.95988281249998</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1145,10 +1145,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1157,13 +1157,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>214.399658203125</v>
+        <v>273.91962890625</v>
       </c>
       <c r="H4">
-        <v>214.519775390625</v>
+        <v>245.250263671875</v>
       </c>
       <c r="I4">
-        <v>-0.1201171875</v>
+        <v>28.66936523437502</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1186,16 +1186,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>211.560302734375</v>
+        <v>259.010302734375</v>
       </c>
       <c r="H5">
-        <v>231.2998046875</v>
+        <v>290.8298046875</v>
       </c>
       <c r="I5">
-        <v>-19.739501953125</v>
+        <v>-31.81950195312498</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1251,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>245.68994140625</v>
+        <v>286.77958984375</v>
       </c>
       <c r="H2">
-        <v>228.189697265625</v>
+        <v>297.5998046875</v>
       </c>
       <c r="I2">
-        <v>17.500244140625</v>
+        <v>-10.82021484375002</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1292,16 +1292,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>235.07958984375</v>
+        <v>294.48994140625</v>
       </c>
       <c r="H3">
-        <v>248.7998046875</v>
+        <v>279.889697265625</v>
       </c>
       <c r="I3">
-        <v>-13.72021484375</v>
+        <v>14.60024414062502</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1327,13 +1327,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>248.11962890625</v>
+        <v>251.320166015625</v>
       </c>
       <c r="H4">
-        <v>234.85986328125</v>
+        <v>251.8599609375</v>
       </c>
       <c r="I4">
-        <v>13.259765625</v>
+        <v>-0.539794921875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>216.420166015625</v>
+        <v>266.51962890625</v>
       </c>
       <c r="H5">
-        <v>233.4599609375</v>
+        <v>269.75986328125</v>
       </c>
       <c r="I5">
-        <v>-17.039794921875</v>
+        <v>-3.240234375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1421,10 +1421,10 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>246.5</v>
+        <v>291.1</v>
       </c>
       <c r="H2">
-        <v>224.349853515625</v>
+        <v>261.449853515625</v>
       </c>
       <c r="I2">
-        <v>22.150146484375</v>
+        <v>29.650146484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1462,16 +1462,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>233.090087890625</v>
+        <v>270.85955078125</v>
       </c>
       <c r="H3">
-        <v>227.58984375</v>
+        <v>285.909912109375</v>
       </c>
       <c r="I3">
-        <v>5.500244140625</v>
+        <v>-15.05036132812501</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1485,10 +1485,10 @@
         <v>38</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1497,13 +1497,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>226.78955078125</v>
+        <v>270.190087890625</v>
       </c>
       <c r="H4">
-        <v>247.159912109375</v>
+        <v>272.18984375</v>
       </c>
       <c r="I4">
-        <v>-20.370361328125</v>
+        <v>-1.999755859375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1526,16 +1526,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>209.619873046875</v>
+        <v>248.369873046875</v>
       </c>
       <c r="H5">
-        <v>216.89990234375</v>
+        <v>260.96990234375</v>
       </c>
       <c r="I5">
-        <v>-7.280029296875</v>
+        <v>-12.60002929687499</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,10 +1591,10 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1603,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>233.83984375</v>
+        <v>279.18984375</v>
       </c>
       <c r="H2">
-        <v>214.35986328125</v>
+        <v>255.85986328125</v>
       </c>
       <c r="I2">
-        <v>19.47998046875</v>
+        <v>23.32998046875002</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1632,16 +1632,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>236.51953125</v>
+        <v>294.7899609375</v>
       </c>
       <c r="H3">
-        <v>215.0400390625</v>
+        <v>276.65966796875</v>
       </c>
       <c r="I3">
-        <v>21.4794921875</v>
+        <v>18.13029296874998</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1655,10 +1655,10 @@
         <v>43</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1667,13 +1667,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>220.9599609375</v>
+        <v>278.01953125</v>
       </c>
       <c r="H4">
-        <v>243.15966796875</v>
+        <v>260.3900390625</v>
       </c>
       <c r="I4">
-        <v>-22.19970703125</v>
+        <v>17.62949218749998</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>209.06005859375</v>
+        <v>242.56005859375</v>
       </c>
       <c r="H5">
-        <v>227.81982421875</v>
+        <v>301.64982421875</v>
       </c>
       <c r="I5">
-        <v>-18.759765625</v>
+        <v>-59.08976562499998</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1761,10 +1761,10 @@
         <v>46</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1773,13 +1773,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>256</v>
+        <v>262.639951171875</v>
       </c>
       <c r="H2">
-        <v>241.52001953125</v>
+        <v>255.60029296875</v>
       </c>
       <c r="I2">
-        <v>14.47998046875</v>
+        <v>7.039658203124986</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>211.449951171875</v>
+        <v>299.8</v>
       </c>
       <c r="H3">
-        <v>211.80029296875</v>
+        <v>292.71001953125</v>
       </c>
       <c r="I3">
-        <v>-0.350341796875</v>
+        <v>7.089980468750014</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1825,10 +1825,10 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1837,13 +1837,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>233.7998046875</v>
+        <v>295.29990234375</v>
       </c>
       <c r="H4">
-        <v>242.489501953125</v>
+        <v>271.88984375</v>
       </c>
       <c r="I4">
-        <v>-8.689697265625</v>
+        <v>23.41005859374997</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1866,16 +1866,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>224.89990234375</v>
+        <v>275.3498046875</v>
       </c>
       <c r="H5">
-        <v>230.33984375</v>
+        <v>312.889501953125</v>
       </c>
       <c r="I5">
-        <v>-5.43994140625</v>
+        <v>-37.53969726562497</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado final da rodada 4
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>282.89029296875</v>
+        <v>282.890380859375</v>
       </c>
       <c r="H2">
-        <v>218.279931640625</v>
+        <v>218.2799072265625</v>
       </c>
       <c r="I2">
-        <v>64.61036132812504</v>
+        <v>64.6104736328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -615,13 +615,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>299.090185546875</v>
+        <v>299.090087890625</v>
       </c>
       <c r="H3">
         <v>259.5703125</v>
       </c>
       <c r="I3">
-        <v>39.51987304687498</v>
+        <v>39.519775390625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -650,10 +650,10 @@
         <v>260.18994140625</v>
       </c>
       <c r="H4">
-        <v>275.04013671875</v>
+        <v>275.0400390625</v>
       </c>
       <c r="I4">
-        <v>-14.85019531249998</v>
+        <v>-14.85009765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>169.630029296875</v>
+        <v>169.6300048828125</v>
       </c>
       <c r="H5">
-        <v>258.910068359375</v>
+        <v>258.91015625</v>
       </c>
       <c r="I5">
-        <v>-89.28003906250004</v>
+        <v>-89.2801513671875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -753,10 +753,10 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>321.41017578125</v>
+        <v>321.41015625</v>
       </c>
       <c r="H2">
-        <v>256.300068359375</v>
+        <v>256.300048828125</v>
       </c>
       <c r="I2">
         <v>65.110107421875</v>
@@ -785,13 +785,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>309.149755859375</v>
+        <v>309.149658203125</v>
       </c>
       <c r="H3">
-        <v>314.0001171875</v>
+        <v>314</v>
       </c>
       <c r="I3">
-        <v>-4.850361328125018</v>
+        <v>-4.850341796875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -817,10 +817,10 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>290.98</v>
+        <v>290.97998046875</v>
       </c>
       <c r="H4">
-        <v>297.579853515625</v>
+        <v>297.579833984375</v>
       </c>
       <c r="I4">
         <v>-6.599853515625</v>
@@ -849,13 +849,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>293.379755859375</v>
+        <v>293.379638671875</v>
       </c>
       <c r="H5">
-        <v>347.0396484375</v>
+        <v>347.03955078125</v>
       </c>
       <c r="I5">
-        <v>-53.65989257812498</v>
+        <v>-53.659912109375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>337.049609375</v>
+        <v>337.0498046875</v>
       </c>
       <c r="H2">
-        <v>292.5197265625</v>
+        <v>292.51953125</v>
       </c>
       <c r="I2">
-        <v>44.52988281249998</v>
+        <v>44.5302734375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -955,13 +955,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>314.65</v>
+        <v>314.64990234375</v>
       </c>
       <c r="H3">
         <v>328.68994140625</v>
       </c>
       <c r="I3">
-        <v>-14.03994140625002</v>
+        <v>-14.0400390625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,13 +987,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>295.3595703125</v>
+        <v>295.359375</v>
       </c>
       <c r="H4">
-        <v>334.649462890625</v>
+        <v>334.649658203125</v>
       </c>
       <c r="I4">
-        <v>-39.28989257812498</v>
+        <v>-39.290283203125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1022,10 +1022,10 @@
         <v>323.249755859375</v>
       </c>
       <c r="H5">
-        <v>314.4498046875</v>
+        <v>314.44970703125</v>
       </c>
       <c r="I5">
-        <v>8.799951171875023</v>
+        <v>8.800048828125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1093,13 +1093,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>279.3001171875</v>
+        <v>279.300048828125</v>
       </c>
       <c r="H2">
         <v>290.10986328125</v>
       </c>
       <c r="I2">
-        <v>-10.80974609374999</v>
+        <v>-10.809814453125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1128,10 +1128,10 @@
         <v>301.86962890625</v>
       </c>
       <c r="H3">
-        <v>271.200263671875</v>
+        <v>271.2001953125</v>
       </c>
       <c r="I3">
-        <v>30.66936523437499</v>
+        <v>30.66943359375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1157,13 +1157,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>300.829658203125</v>
+        <v>300.829833984375</v>
       </c>
       <c r="H4">
-        <v>275.779775390625</v>
+        <v>275.77978515625</v>
       </c>
       <c r="I4">
-        <v>25.04988281250002</v>
+        <v>25.050048828125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1189,13 +1189,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>272.820302734375</v>
+        <v>272.8203125</v>
       </c>
       <c r="H5">
-        <v>317.7298046875</v>
+        <v>317.72998046875</v>
       </c>
       <c r="I5">
-        <v>-44.90950195312502</v>
+        <v>-44.90966796875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>322.72958984375</v>
+        <v>322.7294921875</v>
       </c>
       <c r="H2">
-        <v>319.4998046875</v>
+        <v>319.5</v>
       </c>
       <c r="I2">
-        <v>3.229785156249989</v>
+        <v>3.2294921875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>316.38994140625</v>
+        <v>316.39013671875</v>
       </c>
       <c r="H3">
-        <v>315.839697265625</v>
+        <v>315.839599609375</v>
       </c>
       <c r="I3">
-        <v>0.5502441406250114</v>
+        <v>0.550537109375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1327,13 +1327,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>298.470166015625</v>
+        <v>298.469970703125</v>
       </c>
       <c r="H4">
-        <v>279.1099609375</v>
+        <v>279.10986328125</v>
       </c>
       <c r="I4">
-        <v>19.36020507812503</v>
+        <v>19.360107421875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>293.76962890625</v>
+        <v>293.76953125</v>
       </c>
       <c r="H5">
-        <v>316.90986328125</v>
+        <v>316.90966796875</v>
       </c>
       <c r="I5">
-        <v>-23.14023437500003</v>
+        <v>-23.14013671875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>327.93</v>
+        <v>327.93017578125</v>
       </c>
       <c r="H2">
-        <v>290.999853515625</v>
+        <v>290.999755859375</v>
       </c>
       <c r="I2">
-        <v>36.93014648437503</v>
+        <v>36.930419921875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>299.740087890625</v>
+        <v>299.739990234375</v>
       </c>
       <c r="H3">
-        <v>309.01984375</v>
+        <v>309.02001953125</v>
       </c>
       <c r="I3">
-        <v>-9.27975585937503</v>
+        <v>-9.280029296875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1497,13 +1497,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>292.769873046875</v>
+        <v>292.769775390625</v>
       </c>
       <c r="H4">
-        <v>268.82990234375</v>
+        <v>268.829833984375</v>
       </c>
       <c r="I4">
-        <v>23.93997070312497</v>
+        <v>23.93994140625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1529,13 +1529,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>278.71955078125</v>
+        <v>278.719482421875</v>
       </c>
       <c r="H5">
-        <v>330.309912109375</v>
+        <v>330.309814453125</v>
       </c>
       <c r="I5">
-        <v>-51.59036132812497</v>
+        <v>-51.59033203125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>301.56953125</v>
+        <v>301.5693359375</v>
       </c>
       <c r="H2">
-        <v>268.1900390625</v>
+        <v>268.18994140625</v>
       </c>
       <c r="I2">
-        <v>33.37949218750003</v>
+        <v>33.37939453125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>286.98984375</v>
+        <v>286.98974609375</v>
       </c>
       <c r="H3">
-        <v>279.40986328125</v>
+        <v>279.40966796875</v>
       </c>
       <c r="I3">
-        <v>7.579980468749966</v>
+        <v>7.580078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1667,13 +1667,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>306.9399609375</v>
+        <v>306.93994140625</v>
       </c>
       <c r="H4">
         <v>300.40966796875</v>
       </c>
       <c r="I4">
-        <v>6.530292968750018</v>
+        <v>6.5302734375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1702,10 +1702,10 @@
         <v>266.31005859375</v>
       </c>
       <c r="H5">
-        <v>313.79982421875</v>
+        <v>313.7998046875</v>
       </c>
       <c r="I5">
-        <v>-47.48976562500002</v>
+        <v>-47.48974609375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1773,13 +1773,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>288.709951171875</v>
+        <v>288.709716796875</v>
       </c>
       <c r="H2">
-        <v>276.95029296875</v>
+        <v>276.9501953125</v>
       </c>
       <c r="I2">
-        <v>11.75965820312501</v>
+        <v>11.759521484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>321.15</v>
+        <v>321.14990234375</v>
       </c>
       <c r="H3">
-        <v>318.78001953125</v>
+        <v>318.77978515625</v>
       </c>
       <c r="I3">
-        <v>2.369980468749986</v>
+        <v>2.3701171875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>2</v>
       </c>
       <c r="G4">
-        <v>305.25990234375</v>
+        <v>305.259765625</v>
       </c>
       <c r="H4">
-        <v>304.88984375</v>
+        <v>304.8896484375</v>
       </c>
       <c r="I4">
-        <v>0.3700585937500023</v>
+        <v>0.3701171875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1869,13 +1869,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>308.3498046875</v>
+        <v>308.349609375</v>
       </c>
       <c r="H5">
-        <v>322.849501953125</v>
+        <v>322.849365234375</v>
       </c>
       <c r="I5">
-        <v>-14.499697265625</v>
+        <v>-14.499755859375</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza parciais da rodada 5
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -74,12 +74,12 @@
     <t>Dom Camillo68</t>
   </si>
   <si>
+    <t>S.E.R. GRILLO</t>
+  </si>
+  <si>
     <t>LISI GREMISTA</t>
   </si>
   <si>
-    <t>S.E.R. GRILLO</t>
-  </si>
-  <si>
     <t>Máquina Laranjja</t>
   </si>
   <si>
@@ -101,15 +101,15 @@
     <t>Grupo D</t>
   </si>
   <si>
+    <t>FBC Colorado</t>
+  </si>
+  <si>
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
-    <t>FBC Colorado</t>
-  </si>
-  <si>
     <t>Grêmio imortal 36</t>
   </si>
   <si>
@@ -146,10 +146,10 @@
     <t>Grupo G</t>
   </si>
   <si>
+    <t>Tabajara de Inhaua PB1</t>
+  </si>
+  <si>
     <t>TORRESMO COM PINGA PRO26.1</t>
-  </si>
-  <si>
-    <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
     <t>Grêmio imortal 37</t>
@@ -571,10 +571,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>282.890380859375</v>
+        <v>303.590380859375</v>
       </c>
       <c r="H2">
-        <v>218.2799072265625</v>
+        <v>232.0799072265625</v>
       </c>
       <c r="I2">
-        <v>64.6104736328125</v>
+        <v>71.51047363281248</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>299.090087890625</v>
+        <v>312.890087890625</v>
       </c>
       <c r="H3">
-        <v>259.5703125</v>
+        <v>280.2703125</v>
       </c>
       <c r="I3">
-        <v>39.519775390625</v>
+        <v>32.61977539062502</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -644,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>260.18994140625</v>
+        <v>266.28994140625</v>
       </c>
       <c r="H4">
-        <v>275.0400390625</v>
+        <v>293.1900390625</v>
       </c>
       <c r="I4">
-        <v>-14.85009765625</v>
+        <v>-26.90009765624995</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -667,10 +667,10 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -679,13 +679,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>169.6300048828125</v>
+        <v>187.7800048828125</v>
       </c>
       <c r="H5">
-        <v>258.91015625</v>
+        <v>265.01015625</v>
       </c>
       <c r="I5">
-        <v>-89.2801513671875</v>
+        <v>-77.23015136718752</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -750,16 +750,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>321.41015625</v>
+        <v>335.31015625</v>
       </c>
       <c r="H2">
-        <v>256.300048828125</v>
+        <v>270.600048828125</v>
       </c>
       <c r="I2">
-        <v>65.110107421875</v>
+        <v>64.71010742187497</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -773,10 +773,10 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -785,13 +785,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>309.149658203125</v>
+        <v>302.27998046875</v>
       </c>
       <c r="H3">
-        <v>314</v>
+        <v>306.879833984375</v>
       </c>
       <c r="I3">
-        <v>-4.850341796875</v>
+        <v>-4.599853515625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -814,16 +814,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>290.97998046875</v>
+        <v>318.449658203125</v>
       </c>
       <c r="H4">
-        <v>297.579833984375</v>
+        <v>325.3</v>
       </c>
       <c r="I4">
-        <v>-6.599853515625</v>
+        <v>-6.850341796875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,10 +837,10 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -849,13 +849,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>293.379638671875</v>
+        <v>307.679638671875</v>
       </c>
       <c r="H5">
-        <v>347.03955078125</v>
+        <v>360.93955078125</v>
       </c>
       <c r="I5">
-        <v>-53.659912109375</v>
+        <v>-53.25991210937497</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -911,10 +911,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>337.0498046875</v>
+        <v>378.6498046875</v>
       </c>
       <c r="H2">
-        <v>292.51953125</v>
+        <v>313.11953125</v>
       </c>
       <c r="I2">
-        <v>44.5302734375</v>
+        <v>65.5302734375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -943,10 +943,10 @@
         <v>22</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -955,13 +955,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>314.64990234375</v>
+        <v>336.94990234375</v>
       </c>
       <c r="H3">
-        <v>328.68994140625</v>
+        <v>336.38994140625</v>
       </c>
       <c r="I3">
-        <v>-14.0400390625</v>
+        <v>0.5599609375000227</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -984,16 +984,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>295.359375</v>
+        <v>303.059375</v>
       </c>
       <c r="H4">
-        <v>334.649658203125</v>
+        <v>356.949658203125</v>
       </c>
       <c r="I4">
-        <v>-39.290283203125</v>
+        <v>-53.89028320312502</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1016,16 +1016,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>323.249755859375</v>
+        <v>343.849755859375</v>
       </c>
       <c r="H5">
-        <v>314.44970703125</v>
+        <v>356.04970703125</v>
       </c>
       <c r="I5">
-        <v>8.800048828125</v>
+        <v>-12.199951171875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>279.300048828125</v>
+        <v>326.529833984375</v>
       </c>
       <c r="H2">
-        <v>290.10986328125</v>
+        <v>291.27978515625</v>
       </c>
       <c r="I2">
-        <v>-10.809814453125</v>
+        <v>35.25004882812499</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,10 +1113,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1125,13 +1125,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>301.86962890625</v>
+        <v>294.800048828125</v>
       </c>
       <c r="H3">
-        <v>271.2001953125</v>
+        <v>315.80986328125</v>
       </c>
       <c r="I3">
-        <v>30.66943359375</v>
+        <v>-21.00981445312499</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1154,16 +1154,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>300.829833984375</v>
+        <v>322.76962890625</v>
       </c>
       <c r="H4">
-        <v>275.77978515625</v>
+        <v>303.2001953125</v>
       </c>
       <c r="I4">
-        <v>25.050048828125</v>
+        <v>19.56943359374998</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1177,10 +1177,10 @@
         <v>29</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1189,13 +1189,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>272.8203125</v>
+        <v>304.8203125</v>
       </c>
       <c r="H5">
-        <v>317.72998046875</v>
+        <v>338.62998046875</v>
       </c>
       <c r="I5">
-        <v>-44.90966796875</v>
+        <v>-33.80966796874998</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1251,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>322.7294921875</v>
+        <v>333.2294921875</v>
       </c>
       <c r="H2">
-        <v>319.5</v>
+        <v>328.8</v>
       </c>
       <c r="I2">
-        <v>3.2294921875</v>
+        <v>4.429492187499989</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1283,10 +1283,10 @@
         <v>32</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1295,13 +1295,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>316.39013671875</v>
+        <v>366.89013671875</v>
       </c>
       <c r="H3">
-        <v>315.839599609375</v>
+        <v>330.739599609375</v>
       </c>
       <c r="I3">
-        <v>0.550537109375</v>
+        <v>36.15053710937502</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1324,16 +1324,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>298.469970703125</v>
+        <v>307.769970703125</v>
       </c>
       <c r="H4">
-        <v>279.10986328125</v>
+        <v>289.60986328125</v>
       </c>
       <c r="I4">
-        <v>19.360107421875</v>
+        <v>18.16010742187501</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>293.76953125</v>
+        <v>308.66953125</v>
       </c>
       <c r="H5">
-        <v>316.90966796875</v>
+        <v>367.40966796875</v>
       </c>
       <c r="I5">
-        <v>-23.14013671875</v>
+        <v>-58.74013671875002</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1430,16 +1430,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>327.93017578125</v>
+        <v>339.63017578125</v>
       </c>
       <c r="H2">
-        <v>290.999755859375</v>
+        <v>313.199755859375</v>
       </c>
       <c r="I2">
-        <v>36.930419921875</v>
+        <v>26.430419921875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1453,10 +1453,10 @@
         <v>37</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1465,13 +1465,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>299.739990234375</v>
+        <v>320.139990234375</v>
       </c>
       <c r="H3">
-        <v>309.02001953125</v>
+        <v>323.32001953125</v>
       </c>
       <c r="I3">
-        <v>-9.280029296875</v>
+        <v>-3.180029296875034</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1494,16 +1494,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>292.769775390625</v>
+        <v>307.069775390625</v>
       </c>
       <c r="H4">
-        <v>268.829833984375</v>
+        <v>289.229833984375</v>
       </c>
       <c r="I4">
-        <v>23.93994140625</v>
+        <v>17.83994140625003</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1517,10 +1517,10 @@
         <v>39</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1529,13 +1529,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>278.719482421875</v>
+        <v>300.919482421875</v>
       </c>
       <c r="H5">
-        <v>330.309814453125</v>
+        <v>342.009814453125</v>
       </c>
       <c r="I5">
-        <v>-51.59033203125</v>
+        <v>-41.09033203125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,10 +1591,10 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>301.5693359375</v>
+        <v>334.78974609375</v>
       </c>
       <c r="H2">
-        <v>268.18994140625</v>
+        <v>306.50966796875</v>
       </c>
       <c r="I2">
-        <v>33.37939453125</v>
+        <v>28.28007812499999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1623,10 +1623,10 @@
         <v>42</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>286.98974609375</v>
+        <v>312.0693359375</v>
       </c>
       <c r="H3">
-        <v>279.40966796875</v>
+        <v>272.38994140625</v>
       </c>
       <c r="I3">
-        <v>7.580078125</v>
+        <v>39.67939453125001</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1664,16 +1664,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>306.93994140625</v>
+        <v>334.03994140625</v>
       </c>
       <c r="H4">
-        <v>300.40966796875</v>
+        <v>348.20966796875</v>
       </c>
       <c r="I4">
-        <v>6.5302734375</v>
+        <v>-14.16972656249999</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>266.31005859375</v>
+        <v>270.51005859375</v>
       </c>
       <c r="H5">
-        <v>313.7998046875</v>
+        <v>324.2998046875</v>
       </c>
       <c r="I5">
-        <v>-47.48974609375</v>
+        <v>-53.78974609375001</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1761,10 +1761,10 @@
         <v>46</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1773,13 +1773,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>288.709716796875</v>
+        <v>308.879716796875</v>
       </c>
       <c r="H2">
-        <v>276.9501953125</v>
+        <v>288.2501953125</v>
       </c>
       <c r="I2">
-        <v>11.759521484375</v>
+        <v>20.629521484375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1793,10 +1793,10 @@
         <v>47</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1805,13 +1805,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>321.14990234375</v>
+        <v>343.44990234375</v>
       </c>
       <c r="H3">
-        <v>318.77978515625</v>
+        <v>337.47978515625</v>
       </c>
       <c r="I3">
-        <v>2.3701171875</v>
+        <v>5.970117187500023</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1834,16 +1834,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>305.259765625</v>
+        <v>316.559765625</v>
       </c>
       <c r="H4">
-        <v>304.8896484375</v>
+        <v>325.0596484375</v>
       </c>
       <c r="I4">
-        <v>0.3701171875</v>
+        <v>-8.499882812500005</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1866,16 +1866,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>308.349609375</v>
+        <v>327.049609375</v>
       </c>
       <c r="H5">
-        <v>322.849365234375</v>
+        <v>345.149365234375</v>
       </c>
       <c r="I5">
-        <v>-14.499755859375</v>
+        <v>-18.09975585937502</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Resultado Final da Rodada 5
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -56,12 +56,12 @@
     <t>Grupo A</t>
   </si>
   <si>
+    <t>JV5 Tricolor Gaúcho</t>
+  </si>
+  <si>
     <t>Tatols Beants F.C</t>
   </si>
   <si>
-    <t>JV5 Tricolor Gaúcho</t>
-  </si>
-  <si>
     <t>JUV. KP</t>
   </si>
   <si>
@@ -74,12 +74,12 @@
     <t>Dom Camillo68</t>
   </si>
   <si>
+    <t>LISI GREMISTA</t>
+  </si>
+  <si>
     <t>S.E.R. GRILLO</t>
   </si>
   <si>
-    <t>LISI GREMISTA</t>
-  </si>
-  <si>
     <t>Máquina Laranjja</t>
   </si>
   <si>
@@ -101,12 +101,12 @@
     <t>Grupo D</t>
   </si>
   <si>
+    <t>A Lenda Super Vasco F.c</t>
+  </si>
+  <si>
     <t>FBC Colorado</t>
   </si>
   <si>
-    <t>A Lenda Super Vasco F.c</t>
-  </si>
-  <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
@@ -134,24 +134,24 @@
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>AZURRA82</t>
+  </si>
+  <si>
     <t>DM Studio</t>
   </si>
   <si>
-    <t>AZURRA82</t>
-  </si>
-  <si>
     <t>Rolo Compressor ZN</t>
   </si>
   <si>
     <t>Grupo G</t>
   </si>
   <si>
+    <t>TORRESMO COM PINGA PRO26.1</t>
+  </si>
+  <si>
     <t>Tabajara de Inhaua PB1</t>
   </si>
   <si>
-    <t>TORRESMO COM PINGA PRO26.1</t>
-  </si>
-  <si>
     <t>Grêmio imortal 37</t>
   </si>
   <si>
@@ -161,13 +161,13 @@
     <t>Grupo H</t>
   </si>
   <si>
+    <t>TEAM LOPES 99</t>
+  </si>
+  <si>
     <t>Gremiomaniasm</t>
   </si>
   <si>
     <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>TEAM LOPES 99</t>
   </si>
   <si>
     <t>Super Vasco f.c</t>
@@ -571,25 +571,25 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>303.590380859375</v>
+        <v>383.909912109375</v>
       </c>
       <c r="H2">
-        <v>232.0799072265625</v>
+        <v>340.740234375</v>
       </c>
       <c r="I2">
-        <v>71.51047363281248</v>
+        <v>43.169677734375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -603,25 +603,25 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>312.890087890625</v>
+        <v>364.060302734375</v>
       </c>
       <c r="H3">
-        <v>280.2703125</v>
+        <v>303.0997314453125</v>
       </c>
       <c r="I3">
-        <v>32.61977539062502</v>
+        <v>60.9605712890625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -647,13 +647,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>266.28994140625</v>
+        <v>343.10986328125</v>
       </c>
       <c r="H4">
-        <v>293.1900390625</v>
+        <v>358.4501953125</v>
       </c>
       <c r="I4">
-        <v>-26.90009765624995</v>
+        <v>-15.34033203125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>187.7800048828125</v>
+        <v>253.0401611328125</v>
       </c>
       <c r="H5">
-        <v>265.01015625</v>
+        <v>341.830078125</v>
       </c>
       <c r="I5">
-        <v>-77.23015136718752</v>
+        <v>-88.7899169921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -741,25 +741,25 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>335.31015625</v>
+        <v>406.02001953125</v>
       </c>
       <c r="H2">
-        <v>270.600048828125</v>
+        <v>333.770263671875</v>
       </c>
       <c r="I2">
-        <v>64.71010742187497</v>
+        <v>72.249755859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -785,13 +785,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>302.27998046875</v>
+        <v>383.469482421875</v>
       </c>
       <c r="H3">
-        <v>306.879833984375</v>
+        <v>384.60009765625</v>
       </c>
       <c r="I3">
-        <v>-4.599853515625</v>
+        <v>-1.130615234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -817,13 +817,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>318.449658203125</v>
+        <v>361.580078125</v>
       </c>
       <c r="H4">
-        <v>325.3</v>
+        <v>371.899658203125</v>
       </c>
       <c r="I4">
-        <v>-6.850341796875</v>
+        <v>-10.319580078125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,25 +837,25 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>307.679638671875</v>
+        <v>370.849853515625</v>
       </c>
       <c r="H5">
-        <v>360.93955078125</v>
+        <v>431.6494140625</v>
       </c>
       <c r="I5">
-        <v>-53.25991210937497</v>
+        <v>-60.799560546875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>378.6498046875</v>
+        <v>440.9697265625</v>
       </c>
       <c r="H2">
-        <v>313.11953125</v>
+        <v>373.98974609375</v>
       </c>
       <c r="I2">
-        <v>65.5302734375</v>
+        <v>66.97998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -955,13 +955,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>336.94990234375</v>
+        <v>407.669921875</v>
       </c>
       <c r="H3">
-        <v>336.38994140625</v>
+        <v>411.31005859375</v>
       </c>
       <c r="I3">
-        <v>0.5599609375000227</v>
+        <v>-3.64013671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>303.059375</v>
+        <v>377.9794921875</v>
       </c>
       <c r="H4">
-        <v>356.949658203125</v>
+        <v>427.669677734375</v>
       </c>
       <c r="I4">
-        <v>-53.89028320312502</v>
+        <v>-49.690185546875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1019,13 +1019,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>343.849755859375</v>
+        <v>404.719970703125</v>
       </c>
       <c r="H5">
-        <v>356.04970703125</v>
+        <v>418.36962890625</v>
       </c>
       <c r="I5">
-        <v>-12.199951171875</v>
+        <v>-13.649658203125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1081,25 +1081,25 @@
         <v>26</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>326.529833984375</v>
+        <v>373.920166015625</v>
       </c>
       <c r="H2">
-        <v>291.27978515625</v>
+        <v>376.52978515625</v>
       </c>
       <c r="I2">
-        <v>35.25004882812499</v>
+        <v>-2.609619140625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,25 +1113,25 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>294.800048828125</v>
+        <v>387.249755859375</v>
       </c>
       <c r="H3">
-        <v>315.80986328125</v>
+        <v>370.39990234375</v>
       </c>
       <c r="I3">
-        <v>-21.00981445312499</v>
+        <v>16.849853515625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1157,13 +1157,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>322.76962890625</v>
+        <v>385.189453125</v>
       </c>
       <c r="H4">
-        <v>303.2001953125</v>
+        <v>361.5703125</v>
       </c>
       <c r="I4">
-        <v>19.56943359374998</v>
+        <v>23.619140625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1189,13 +1189,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>304.8203125</v>
+        <v>363.1904296875</v>
       </c>
       <c r="H5">
-        <v>338.62998046875</v>
+        <v>401.0498046875</v>
       </c>
       <c r="I5">
-        <v>-33.80966796874998</v>
+        <v>-37.859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>333.2294921875</v>
+        <v>411.74951171875</v>
       </c>
       <c r="H2">
-        <v>328.8</v>
+        <v>397.419921875</v>
       </c>
       <c r="I2">
-        <v>4.429492187499989</v>
+        <v>14.32958984375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>366.89013671875</v>
+        <v>419.9599609375</v>
       </c>
       <c r="H3">
-        <v>330.739599609375</v>
+        <v>388.109619140625</v>
       </c>
       <c r="I3">
-        <v>36.15053710937502</v>
+        <v>31.850341796875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1327,13 +1327,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>307.769970703125</v>
+        <v>376.389892578125</v>
       </c>
       <c r="H4">
-        <v>289.60986328125</v>
+        <v>368.1298828125</v>
       </c>
       <c r="I4">
-        <v>18.16010742187501</v>
+        <v>8.260009765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>308.66953125</v>
+        <v>366.03955078125</v>
       </c>
       <c r="H5">
-        <v>367.40966796875</v>
+        <v>420.4794921875</v>
       </c>
       <c r="I5">
-        <v>-58.74013671875002</v>
+        <v>-54.43994140625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1421,25 +1421,25 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>339.63017578125</v>
+        <v>413.60009765625</v>
       </c>
       <c r="H2">
-        <v>313.199755859375</v>
+        <v>365.769775390625</v>
       </c>
       <c r="I2">
-        <v>26.430419921875</v>
+        <v>47.830322265625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>320.139990234375</v>
+        <v>370.239990234375</v>
       </c>
       <c r="H3">
-        <v>323.32001953125</v>
+        <v>337.939697265625</v>
       </c>
       <c r="I3">
-        <v>-3.180029296875034</v>
+        <v>32.30029296875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1497,13 +1497,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>307.069775390625</v>
+        <v>368.849853515625</v>
       </c>
       <c r="H4">
-        <v>289.229833984375</v>
+        <v>386.490234375</v>
       </c>
       <c r="I4">
-        <v>17.83994140625003</v>
+        <v>-17.640380859375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1517,25 +1517,25 @@
         <v>39</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>300.919482421875</v>
+        <v>353.489501953125</v>
       </c>
       <c r="H5">
-        <v>342.009814453125</v>
+        <v>415.979736328125</v>
       </c>
       <c r="I5">
-        <v>-41.09033203125</v>
+        <v>-62.490234375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>334.78974609375</v>
+        <v>397.189453125</v>
       </c>
       <c r="H2">
-        <v>306.50966796875</v>
+        <v>347.7099609375</v>
       </c>
       <c r="I2">
-        <v>28.28007812499999</v>
+        <v>49.4794921875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>312.0693359375</v>
+        <v>374.509765625</v>
       </c>
       <c r="H3">
-        <v>272.38994140625</v>
+        <v>366.6298828125</v>
       </c>
       <c r="I3">
-        <v>39.67939453125001</v>
+        <v>7.8798828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1667,13 +1667,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>334.03994140625</v>
+        <v>394.16015625</v>
       </c>
       <c r="H4">
-        <v>348.20966796875</v>
+        <v>387.9296875</v>
       </c>
       <c r="I4">
-        <v>-14.16972656249999</v>
+        <v>6.23046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1699,13 +1699,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>270.51005859375</v>
+        <v>345.830078125</v>
       </c>
       <c r="H5">
-        <v>324.2998046875</v>
+        <v>409.419921875</v>
       </c>
       <c r="I5">
-        <v>-53.78974609375001</v>
+        <v>-63.58984375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1761,25 +1761,25 @@
         <v>46</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>308.879716796875</v>
+        <v>403.77978515625</v>
       </c>
       <c r="H2">
-        <v>288.2501953125</v>
+        <v>374.259765625</v>
       </c>
       <c r="I2">
-        <v>20.629521484375</v>
+        <v>29.52001953125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>343.44990234375</v>
+        <v>358.079833984375</v>
       </c>
       <c r="H3">
-        <v>337.47978515625</v>
+        <v>375.47021484375</v>
       </c>
       <c r="I3">
-        <v>5.970117187500023</v>
+        <v>-17.390380859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>316.559765625</v>
+        <v>414.169921875</v>
       </c>
       <c r="H4">
-        <v>325.0596484375</v>
+        <v>414.89990234375</v>
       </c>
       <c r="I4">
-        <v>-8.499882812500005</v>
+        <v>-0.72998046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1857,25 +1857,25 @@
         <v>49</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>327.049609375</v>
+        <v>404.4697265625</v>
       </c>
       <c r="H5">
-        <v>345.149365234375</v>
+        <v>415.869384765625</v>
       </c>
       <c r="I5">
-        <v>-18.09975585937502</v>
+        <v>-11.399658203125</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Atualiza parciais da Rodada 6
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -77,12 +77,12 @@
     <t>LISI GREMISTA</t>
   </si>
   <si>
+    <t>Máquina Laranjja</t>
+  </si>
+  <si>
     <t>S.E.R. GRILLO</t>
   </si>
   <si>
-    <t>Máquina Laranjja</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
@@ -104,15 +104,15 @@
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
+    <t>Mau Humor F.C.</t>
+  </si>
+  <si>
+    <t>Grêmio imortal 36</t>
+  </si>
+  <si>
     <t>FBC Colorado</t>
   </si>
   <si>
-    <t>Mau Humor F.C.</t>
-  </si>
-  <si>
-    <t>Grêmio imortal 36</t>
-  </si>
-  <si>
     <t>Grupo E</t>
   </si>
   <si>
@@ -134,12 +134,12 @@
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>DM Studio</t>
+  </si>
+  <si>
     <t>AZURRA82</t>
   </si>
   <si>
-    <t>DM Studio</t>
-  </si>
-  <si>
     <t>Rolo Compressor ZN</t>
   </si>
   <si>
@@ -161,16 +161,16 @@
     <t>Grupo H</t>
   </si>
   <si>
+    <t>Texas Club 2026</t>
+  </si>
+  <si>
     <t>TEAM LOPES 99</t>
   </si>
   <si>
+    <t>Super Vasco f.c</t>
+  </si>
+  <si>
     <t>Gremiomaniasm</t>
-  </si>
-  <si>
-    <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>Super Vasco f.c</t>
   </si>
 </sst>
 </file>
@@ -571,10 +571,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>383.909912109375</v>
+        <v>445.919912109375</v>
       </c>
       <c r="H2">
-        <v>340.740234375</v>
+        <v>388.940234375</v>
       </c>
       <c r="I2">
-        <v>43.169677734375</v>
+        <v>56.979677734375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -603,10 +603,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>364.060302734375</v>
+        <v>426.980302734375</v>
       </c>
       <c r="H3">
-        <v>303.0997314453125</v>
+        <v>357.3097314453125</v>
       </c>
       <c r="I3">
-        <v>60.9605712890625</v>
+        <v>69.67057128906254</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -644,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>343.10986328125</v>
+        <v>397.31986328125</v>
       </c>
       <c r="H4">
-        <v>358.4501953125</v>
+        <v>421.3701953125</v>
       </c>
       <c r="I4">
-        <v>-15.34033203125</v>
+        <v>-24.05033203125004</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -676,16 +676,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>253.0401611328125</v>
+        <v>301.2401611328125</v>
       </c>
       <c r="H5">
-        <v>341.830078125</v>
+        <v>403.840078125</v>
       </c>
       <c r="I5">
-        <v>-88.7899169921875</v>
+        <v>-102.5999169921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>406.02001953125</v>
+        <v>478.13001953125</v>
       </c>
       <c r="H2">
-        <v>333.770263671875</v>
+        <v>398.130263671875</v>
       </c>
       <c r="I2">
-        <v>72.249755859375</v>
+        <v>79.999755859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>383.469482421875</v>
+        <v>447.829482421875</v>
       </c>
       <c r="H3">
-        <v>384.60009765625</v>
+        <v>456.71009765625</v>
       </c>
       <c r="I3">
-        <v>-1.130615234375</v>
+        <v>-8.880615234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -814,16 +814,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>361.580078125</v>
+        <v>434.969853515625</v>
       </c>
       <c r="H4">
-        <v>371.899658203125</v>
+        <v>476.1594140625</v>
       </c>
       <c r="I4">
-        <v>-10.319580078125</v>
+        <v>-41.18956054687499</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,10 +837,10 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -849,13 +849,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>370.849853515625</v>
+        <v>406.090078125</v>
       </c>
       <c r="H5">
-        <v>431.6494140625</v>
+        <v>436.019658203125</v>
       </c>
       <c r="I5">
-        <v>-60.799560546875</v>
+        <v>-29.92958007812501</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -911,10 +911,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>440.9697265625</v>
+        <v>527.3897265625</v>
       </c>
       <c r="H2">
-        <v>373.98974609375</v>
+        <v>456.98974609375</v>
       </c>
       <c r="I2">
-        <v>66.97998046875</v>
+        <v>70.39998046874996</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>407.669921875</v>
+        <v>490.669921875</v>
       </c>
       <c r="H3">
-        <v>411.31005859375</v>
+        <v>497.73005859375</v>
       </c>
       <c r="I3">
-        <v>-3.64013671875</v>
+        <v>-7.060136718750016</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -975,10 +975,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -987,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>377.9794921875</v>
+        <v>444.5894921875</v>
       </c>
       <c r="H4">
-        <v>427.669677734375</v>
+        <v>484.069677734375</v>
       </c>
       <c r="I4">
-        <v>-49.690185546875</v>
+        <v>-39.48018554687496</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1016,16 +1016,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>404.719970703125</v>
+        <v>461.119970703125</v>
       </c>
       <c r="H5">
-        <v>418.36962890625</v>
+        <v>484.97962890625</v>
       </c>
       <c r="I5">
-        <v>-13.649658203125</v>
+        <v>-23.85965820312504</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>373.920166015625</v>
+        <v>442.720166015625</v>
       </c>
       <c r="H2">
-        <v>376.52978515625</v>
+        <v>448.61978515625</v>
       </c>
       <c r="I2">
-        <v>-2.609619140625</v>
+        <v>-5.89961914062502</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,10 +1113,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1125,13 +1125,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>387.249755859375</v>
+        <v>439.999453125</v>
       </c>
       <c r="H3">
-        <v>370.39990234375</v>
+        <v>408.9603125</v>
       </c>
       <c r="I3">
-        <v>16.849853515625</v>
+        <v>31.03914062500002</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1145,10 +1145,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1157,13 +1157,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>385.189453125</v>
+        <v>435.2804296875</v>
       </c>
       <c r="H4">
-        <v>361.5703125</v>
+        <v>469.8498046875</v>
       </c>
       <c r="I4">
-        <v>23.619140625</v>
+        <v>-34.56937499999998</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1186,16 +1186,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>363.1904296875</v>
+        <v>434.639755859375</v>
       </c>
       <c r="H5">
-        <v>401.0498046875</v>
+        <v>425.20990234375</v>
       </c>
       <c r="I5">
-        <v>-37.859375</v>
+        <v>9.429853515624984</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1251,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>411.74951171875</v>
+        <v>474.55951171875</v>
       </c>
       <c r="H2">
-        <v>397.419921875</v>
+        <v>450.879921875</v>
       </c>
       <c r="I2">
-        <v>14.32958984375</v>
+        <v>23.67958984375002</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1292,16 +1292,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>419.9599609375</v>
+        <v>485.8499609375</v>
       </c>
       <c r="H3">
-        <v>388.109619140625</v>
+        <v>461.329619140625</v>
       </c>
       <c r="I3">
-        <v>31.850341796875</v>
+        <v>24.52034179687496</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1327,13 +1327,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>376.389892578125</v>
+        <v>449.609892578125</v>
       </c>
       <c r="H4">
-        <v>368.1298828125</v>
+        <v>434.0198828125</v>
       </c>
       <c r="I4">
-        <v>8.260009765625</v>
+        <v>15.59000976562504</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>366.03955078125</v>
+        <v>419.49955078125</v>
       </c>
       <c r="H5">
-        <v>420.4794921875</v>
+        <v>483.2894921875</v>
       </c>
       <c r="I5">
-        <v>-54.43994140625</v>
+        <v>-63.78994140625002</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1421,10 +1421,10 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>413.60009765625</v>
+        <v>472.21009765625</v>
       </c>
       <c r="H2">
-        <v>365.769775390625</v>
+        <v>420.389775390625</v>
       </c>
       <c r="I2">
-        <v>47.830322265625</v>
+        <v>51.82032226562501</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1462,16 +1462,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>370.239990234375</v>
+        <v>436.039853515625</v>
       </c>
       <c r="H3">
-        <v>337.939697265625</v>
+        <v>453.000234375</v>
       </c>
       <c r="I3">
-        <v>32.30029296875</v>
+        <v>-16.96038085937499</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1485,10 +1485,10 @@
         <v>38</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1497,13 +1497,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>368.849853515625</v>
+        <v>424.859990234375</v>
       </c>
       <c r="H4">
-        <v>386.490234375</v>
+        <v>396.549697265625</v>
       </c>
       <c r="I4">
-        <v>-17.640380859375</v>
+        <v>28.31029296874999</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1526,16 +1526,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>353.489501953125</v>
+        <v>419.999501953125</v>
       </c>
       <c r="H5">
-        <v>415.979736328125</v>
+        <v>483.169736328125</v>
       </c>
       <c r="I5">
-        <v>-62.490234375</v>
+        <v>-63.17023437500001</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,10 +1591,10 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>397.189453125</v>
+        <v>466.609453125</v>
       </c>
       <c r="H2">
-        <v>347.7099609375</v>
+        <v>409.8099609375</v>
       </c>
       <c r="I2">
-        <v>49.4794921875</v>
+        <v>56.79949218749999</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1623,10 +1623,10 @@
         <v>42</v>
       </c>
       <c r="C3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>374.509765625</v>
+        <v>443.629765625</v>
       </c>
       <c r="H3">
-        <v>366.6298828125</v>
+        <v>422.7398828125</v>
       </c>
       <c r="I3">
-        <v>7.8798828125</v>
+        <v>20.88988281249999</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1664,16 +1664,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>394.16015625</v>
+        <v>456.26015625</v>
       </c>
       <c r="H4">
-        <v>387.9296875</v>
+        <v>457.3496875</v>
       </c>
       <c r="I4">
-        <v>6.23046875</v>
+        <v>-1.089531249999993</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>345.830078125</v>
+        <v>401.940078125</v>
       </c>
       <c r="H5">
-        <v>409.419921875</v>
+        <v>478.539921875</v>
       </c>
       <c r="I5">
-        <v>-63.58984375</v>
+        <v>-76.59984374999999</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1770,16 +1770,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>403.77978515625</v>
+        <v>497.169921875</v>
       </c>
       <c r="H2">
-        <v>374.259765625</v>
+        <v>492.30990234375</v>
       </c>
       <c r="I2">
-        <v>29.52001953125</v>
+        <v>4.860019531250032</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>358.079833984375</v>
+        <v>481.18978515625</v>
       </c>
       <c r="H3">
-        <v>375.47021484375</v>
+        <v>457.259765625</v>
       </c>
       <c r="I3">
-        <v>-17.390380859375</v>
+        <v>23.93001953124997</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1825,10 +1825,10 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1837,13 +1837,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>414.169921875</v>
+        <v>470.1797265625</v>
       </c>
       <c r="H4">
-        <v>414.89990234375</v>
+        <v>468.069384765625</v>
       </c>
       <c r="I4">
-        <v>-0.72998046875</v>
+        <v>2.110341796874991</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1857,10 +1857,10 @@
         <v>49</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1869,13 +1869,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>404.4697265625</v>
+        <v>410.279833984375</v>
       </c>
       <c r="H5">
-        <v>415.869384765625</v>
+        <v>441.18021484375</v>
       </c>
       <c r="I5">
-        <v>-11.399658203125</v>
+        <v>-30.90038085937499</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Ajusta Fase 2 da Libertadores
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -583,13 +583,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>445.919912109375</v>
+        <v>445.919921875</v>
       </c>
       <c r="H2">
-        <v>388.940234375</v>
+        <v>388.940185546875</v>
       </c>
       <c r="I2">
-        <v>56.979677734375</v>
+        <v>56.979736328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -615,13 +615,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>426.980302734375</v>
+        <v>426.980224609375</v>
       </c>
       <c r="H3">
-        <v>357.3097314453125</v>
+        <v>357.3096923828125</v>
       </c>
       <c r="I3">
-        <v>69.67057128906254</v>
+        <v>69.6705322265625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -647,13 +647,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>397.31986328125</v>
+        <v>397.31982421875</v>
       </c>
       <c r="H4">
-        <v>421.3701953125</v>
+        <v>421.3701171875</v>
       </c>
       <c r="I4">
-        <v>-24.05033203125004</v>
+        <v>-24.05029296875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -679,13 +679,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>301.2401611328125</v>
+        <v>301.2401123046875</v>
       </c>
       <c r="H5">
-        <v>403.840078125</v>
+        <v>403.840087890625</v>
       </c>
       <c r="I5">
-        <v>-102.5999169921875</v>
+        <v>-102.5999755859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -753,10 +753,10 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>478.13001953125</v>
+        <v>478.1298828125</v>
       </c>
       <c r="H2">
-        <v>398.130263671875</v>
+        <v>398.130126953125</v>
       </c>
       <c r="I2">
         <v>79.999755859375</v>
@@ -785,10 +785,10 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>447.829482421875</v>
+        <v>447.829345703125</v>
       </c>
       <c r="H3">
-        <v>456.71009765625</v>
+        <v>456.7099609375</v>
       </c>
       <c r="I3">
         <v>-8.880615234375</v>
@@ -817,13 +817,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>434.969853515625</v>
+        <v>434.969970703125</v>
       </c>
       <c r="H4">
-        <v>476.1594140625</v>
+        <v>476.159423828125</v>
       </c>
       <c r="I4">
-        <v>-41.18956054687499</v>
+        <v>-41.189453125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -849,13 +849,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>406.090078125</v>
+        <v>406.090087890625</v>
       </c>
       <c r="H5">
-        <v>436.019658203125</v>
+        <v>436.019775390625</v>
       </c>
       <c r="I5">
-        <v>-29.92958007812501</v>
+        <v>-29.9296875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>527.3897265625</v>
+        <v>527.3896484375</v>
       </c>
       <c r="H2">
         <v>456.98974609375</v>
       </c>
       <c r="I2">
-        <v>70.39998046874996</v>
+        <v>70.39990234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -958,10 +958,10 @@
         <v>490.669921875</v>
       </c>
       <c r="H3">
-        <v>497.73005859375</v>
+        <v>497.72998046875</v>
       </c>
       <c r="I3">
-        <v>-7.060136718750016</v>
+        <v>-7.06005859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -987,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>444.5894921875</v>
+        <v>444.58935546875</v>
       </c>
       <c r="H4">
-        <v>484.069677734375</v>
+        <v>484.069580078125</v>
       </c>
       <c r="I4">
-        <v>-39.48018554687496</v>
+        <v>-39.480224609375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1019,13 +1019,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>461.119970703125</v>
+        <v>461.119873046875</v>
       </c>
       <c r="H5">
-        <v>484.97962890625</v>
+        <v>484.9794921875</v>
       </c>
       <c r="I5">
-        <v>-23.85965820312504</v>
+        <v>-23.859619140625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1093,13 +1093,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>442.720166015625</v>
+        <v>442.719970703125</v>
       </c>
       <c r="H2">
-        <v>448.61978515625</v>
+        <v>448.61962890625</v>
       </c>
       <c r="I2">
-        <v>-5.89961914062502</v>
+        <v>-5.899658203125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1125,13 +1125,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>439.999453125</v>
+        <v>439.99951171875</v>
       </c>
       <c r="H3">
-        <v>408.9603125</v>
+        <v>408.960205078125</v>
       </c>
       <c r="I3">
-        <v>31.03914062500002</v>
+        <v>31.039306640625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1157,13 +1157,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>435.2804296875</v>
+        <v>435.2802734375</v>
       </c>
       <c r="H4">
-        <v>469.8498046875</v>
+        <v>469.849609375</v>
       </c>
       <c r="I4">
-        <v>-34.56937499999998</v>
+        <v>-34.5693359375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1189,13 +1189,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>434.639755859375</v>
+        <v>434.6396484375</v>
       </c>
       <c r="H5">
-        <v>425.20990234375</v>
+        <v>425.2099609375</v>
       </c>
       <c r="I5">
-        <v>9.429853515624984</v>
+        <v>9.4296875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>474.55951171875</v>
+        <v>474.5595703125</v>
       </c>
       <c r="H2">
-        <v>450.879921875</v>
+        <v>450.8798828125</v>
       </c>
       <c r="I2">
-        <v>23.67958984375002</v>
+        <v>23.6796875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1295,13 +1295,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>485.8499609375</v>
+        <v>485.85009765625</v>
       </c>
       <c r="H3">
-        <v>461.329619140625</v>
+        <v>461.329833984375</v>
       </c>
       <c r="I3">
-        <v>24.52034179687496</v>
+        <v>24.520263671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1327,13 +1327,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>449.609892578125</v>
+        <v>449.610107421875</v>
       </c>
       <c r="H4">
-        <v>434.0198828125</v>
+        <v>434.02001953125</v>
       </c>
       <c r="I4">
-        <v>15.59000976562504</v>
+        <v>15.590087890625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1359,13 +1359,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>419.49955078125</v>
+        <v>419.49951171875</v>
       </c>
       <c r="H5">
-        <v>483.2894921875</v>
+        <v>483.28955078125</v>
       </c>
       <c r="I5">
-        <v>-63.78994140625002</v>
+        <v>-63.7900390625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>472.21009765625</v>
+        <v>472.210205078125</v>
       </c>
       <c r="H2">
-        <v>420.389775390625</v>
+        <v>420.389892578125</v>
       </c>
       <c r="I2">
-        <v>51.82032226562501</v>
+        <v>51.8203125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>436.039853515625</v>
+        <v>436.039794921875</v>
       </c>
       <c r="H3">
-        <v>453.000234375</v>
+        <v>453</v>
       </c>
       <c r="I3">
-        <v>-16.96038085937499</v>
+        <v>-16.960205078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1497,13 +1497,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>424.859990234375</v>
+        <v>424.860107421875</v>
       </c>
       <c r="H4">
-        <v>396.549697265625</v>
+        <v>396.5498046875</v>
       </c>
       <c r="I4">
-        <v>28.31029296874999</v>
+        <v>28.310302734375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1529,13 +1529,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>419.999501953125</v>
+        <v>419.999267578125</v>
       </c>
       <c r="H5">
-        <v>483.169736328125</v>
+        <v>483.169677734375</v>
       </c>
       <c r="I5">
-        <v>-63.17023437500001</v>
+        <v>-63.17041015625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>466.609453125</v>
+        <v>466.609375</v>
       </c>
       <c r="H2">
-        <v>409.8099609375</v>
+        <v>409.81005859375</v>
       </c>
       <c r="I2">
-        <v>56.79949218749999</v>
+        <v>56.79931640625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>443.629765625</v>
+        <v>443.6298828125</v>
       </c>
       <c r="H3">
-        <v>422.7398828125</v>
+        <v>422.739990234375</v>
       </c>
       <c r="I3">
-        <v>20.88988281249999</v>
+        <v>20.889892578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1667,13 +1667,13 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <v>456.26015625</v>
+        <v>456.26025390625</v>
       </c>
       <c r="H4">
-        <v>457.3496875</v>
+        <v>457.349609375</v>
       </c>
       <c r="I4">
-        <v>-1.089531249999993</v>
+        <v>-1.08935546875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1699,13 +1699,13 @@
         <v>6</v>
       </c>
       <c r="G5">
-        <v>401.940078125</v>
+        <v>401.940185546875</v>
       </c>
       <c r="H5">
-        <v>478.539921875</v>
+        <v>478.5400390625</v>
       </c>
       <c r="I5">
-        <v>-76.59984374999999</v>
+        <v>-76.599853515625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1776,10 +1776,10 @@
         <v>497.169921875</v>
       </c>
       <c r="H2">
-        <v>492.30990234375</v>
+        <v>492.31005859375</v>
       </c>
       <c r="I2">
-        <v>4.860019531250032</v>
+        <v>4.85986328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1805,13 +1805,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>481.18978515625</v>
+        <v>481.18994140625</v>
       </c>
       <c r="H3">
         <v>457.259765625</v>
       </c>
       <c r="I3">
-        <v>23.93001953124997</v>
+        <v>23.93017578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1837,13 +1837,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>470.1797265625</v>
+        <v>470.1796875</v>
       </c>
       <c r="H4">
-        <v>468.069384765625</v>
+        <v>468.0693359375</v>
       </c>
       <c r="I4">
-        <v>2.110341796874991</v>
+        <v>2.1103515625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1869,13 +1869,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>410.279833984375</v>
+        <v>410.27978515625</v>
       </c>
       <c r="H5">
-        <v>441.18021484375</v>
+        <v>441.18017578125</v>
       </c>
       <c r="I5">
-        <v>-30.90038085937499</v>
+        <v>-30.900390625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Organiza terceiros colocados da fase 1 da Libertadores
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -77,12 +77,12 @@
     <t>LISI GREMISTA</t>
   </si>
   <si>
+    <t>S.E.R. GRILLO</t>
+  </si>
+  <si>
     <t>Máquina Laranjja</t>
   </si>
   <si>
-    <t>S.E.R. GRILLO</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
@@ -104,15 +104,15 @@
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
+    <t>FBC Colorado</t>
+  </si>
+  <si>
     <t>Mau Humor F.C.</t>
   </si>
   <si>
     <t>Grêmio imortal 36</t>
   </si>
   <si>
-    <t>FBC Colorado</t>
-  </si>
-  <si>
     <t>Grupo E</t>
   </si>
   <si>
@@ -134,12 +134,12 @@
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>AZURRA82</t>
+  </si>
+  <si>
     <t>DM Studio</t>
   </si>
   <si>
-    <t>AZURRA82</t>
-  </si>
-  <si>
     <t>Rolo Compressor ZN</t>
   </si>
   <si>
@@ -161,16 +161,16 @@
     <t>Grupo H</t>
   </si>
   <si>
+    <t>TEAM LOPES 99</t>
+  </si>
+  <si>
+    <t>Gremiomaniasm</t>
+  </si>
+  <si>
     <t>Texas Club 2026</t>
   </si>
   <si>
-    <t>TEAM LOPES 99</t>
-  </si>
-  <si>
     <t>Super Vasco f.c</t>
-  </si>
-  <si>
-    <t>Gremiomaniasm</t>
   </si>
 </sst>
 </file>
@@ -571,10 +571,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>445.919921875</v>
+        <v>383.909912109375</v>
       </c>
       <c r="H2">
-        <v>388.940185546875</v>
+        <v>340.740234375</v>
       </c>
       <c r="I2">
-        <v>56.979736328125</v>
+        <v>43.169677734375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -603,10 +603,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>426.980224609375</v>
+        <v>364.060302734375</v>
       </c>
       <c r="H3">
-        <v>357.3096923828125</v>
+        <v>303.0997314453125</v>
       </c>
       <c r="I3">
-        <v>69.6705322265625</v>
+        <v>60.9605712890625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -644,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>397.31982421875</v>
+        <v>343.10986328125</v>
       </c>
       <c r="H4">
-        <v>421.3701171875</v>
+        <v>358.4501953125</v>
       </c>
       <c r="I4">
-        <v>-24.05029296875</v>
+        <v>-15.34033203125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -676,16 +676,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>301.2401123046875</v>
+        <v>253.0401611328125</v>
       </c>
       <c r="H5">
-        <v>403.840087890625</v>
+        <v>341.830078125</v>
       </c>
       <c r="I5">
-        <v>-102.5999755859375</v>
+        <v>-88.7899169921875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>478.1298828125</v>
+        <v>406.02001953125</v>
       </c>
       <c r="H2">
-        <v>398.130126953125</v>
+        <v>333.770263671875</v>
       </c>
       <c r="I2">
-        <v>79.999755859375</v>
+        <v>72.249755859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>447.829345703125</v>
+        <v>383.469482421875</v>
       </c>
       <c r="H3">
-        <v>456.7099609375</v>
+        <v>384.60009765625</v>
       </c>
       <c r="I3">
-        <v>-8.880615234375</v>
+        <v>-1.130615234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -814,16 +814,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>434.969970703125</v>
+        <v>361.580078125</v>
       </c>
       <c r="H4">
-        <v>476.159423828125</v>
+        <v>371.899658203125</v>
       </c>
       <c r="I4">
-        <v>-41.189453125</v>
+        <v>-10.319580078125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,10 +837,10 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -849,13 +849,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>406.090087890625</v>
+        <v>370.849853515625</v>
       </c>
       <c r="H5">
-        <v>436.019775390625</v>
+        <v>431.6494140625</v>
       </c>
       <c r="I5">
-        <v>-29.9296875</v>
+        <v>-60.799560546875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -911,10 +911,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>527.3896484375</v>
+        <v>440.9697265625</v>
       </c>
       <c r="H2">
-        <v>456.98974609375</v>
+        <v>373.98974609375</v>
       </c>
       <c r="I2">
-        <v>70.39990234375</v>
+        <v>66.97998046875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>490.669921875</v>
+        <v>407.669921875</v>
       </c>
       <c r="H3">
-        <v>497.72998046875</v>
+        <v>411.31005859375</v>
       </c>
       <c r="I3">
-        <v>-7.06005859375</v>
+        <v>-3.64013671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -975,10 +975,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -987,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>444.58935546875</v>
+        <v>377.9794921875</v>
       </c>
       <c r="H4">
-        <v>484.069580078125</v>
+        <v>427.669677734375</v>
       </c>
       <c r="I4">
-        <v>-39.480224609375</v>
+        <v>-49.690185546875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1016,16 +1016,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>461.119873046875</v>
+        <v>404.719970703125</v>
       </c>
       <c r="H5">
-        <v>484.9794921875</v>
+        <v>418.36962890625</v>
       </c>
       <c r="I5">
-        <v>-23.859619140625</v>
+        <v>-13.649658203125</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>442.719970703125</v>
+        <v>373.920166015625</v>
       </c>
       <c r="H2">
-        <v>448.61962890625</v>
+        <v>376.52978515625</v>
       </c>
       <c r="I2">
-        <v>-5.899658203125</v>
+        <v>-2.609619140625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,10 +1113,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1125,13 +1125,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>439.99951171875</v>
+        <v>387.249755859375</v>
       </c>
       <c r="H3">
-        <v>408.960205078125</v>
+        <v>370.39990234375</v>
       </c>
       <c r="I3">
-        <v>31.039306640625</v>
+        <v>16.849853515625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1145,10 +1145,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1157,13 +1157,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>435.2802734375</v>
+        <v>385.189453125</v>
       </c>
       <c r="H4">
-        <v>469.849609375</v>
+        <v>361.5703125</v>
       </c>
       <c r="I4">
-        <v>-34.5693359375</v>
+        <v>23.619140625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1186,16 +1186,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>434.6396484375</v>
+        <v>363.1904296875</v>
       </c>
       <c r="H5">
-        <v>425.2099609375</v>
+        <v>401.0498046875</v>
       </c>
       <c r="I5">
-        <v>9.4296875</v>
+        <v>-37.859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1251,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>474.5595703125</v>
+        <v>411.74951171875</v>
       </c>
       <c r="H2">
-        <v>450.8798828125</v>
+        <v>397.419921875</v>
       </c>
       <c r="I2">
-        <v>23.6796875</v>
+        <v>14.32958984375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1292,16 +1292,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>485.85009765625</v>
+        <v>419.9599609375</v>
       </c>
       <c r="H3">
-        <v>461.329833984375</v>
+        <v>388.109619140625</v>
       </c>
       <c r="I3">
-        <v>24.520263671875</v>
+        <v>31.850341796875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1327,13 +1327,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>449.610107421875</v>
+        <v>376.389892578125</v>
       </c>
       <c r="H4">
-        <v>434.02001953125</v>
+        <v>368.1298828125</v>
       </c>
       <c r="I4">
-        <v>15.590087890625</v>
+        <v>8.260009765625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>419.49951171875</v>
+        <v>366.03955078125</v>
       </c>
       <c r="H5">
-        <v>483.28955078125</v>
+        <v>420.4794921875</v>
       </c>
       <c r="I5">
-        <v>-63.7900390625</v>
+        <v>-54.43994140625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1421,10 +1421,10 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>472.210205078125</v>
+        <v>413.60009765625</v>
       </c>
       <c r="H2">
-        <v>420.389892578125</v>
+        <v>365.769775390625</v>
       </c>
       <c r="I2">
-        <v>51.8203125</v>
+        <v>47.830322265625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1462,16 +1462,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>436.039794921875</v>
+        <v>370.239990234375</v>
       </c>
       <c r="H3">
-        <v>453</v>
+        <v>337.939697265625</v>
       </c>
       <c r="I3">
-        <v>-16.960205078125</v>
+        <v>32.30029296875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1485,10 +1485,10 @@
         <v>38</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1497,13 +1497,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>424.860107421875</v>
+        <v>368.849853515625</v>
       </c>
       <c r="H4">
-        <v>396.5498046875</v>
+        <v>386.490234375</v>
       </c>
       <c r="I4">
-        <v>28.310302734375</v>
+        <v>-17.640380859375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1526,16 +1526,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>419.999267578125</v>
+        <v>353.489501953125</v>
       </c>
       <c r="H5">
-        <v>483.169677734375</v>
+        <v>415.979736328125</v>
       </c>
       <c r="I5">
-        <v>-63.17041015625</v>
+        <v>-62.490234375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,10 +1591,10 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>466.609375</v>
+        <v>397.189453125</v>
       </c>
       <c r="H2">
-        <v>409.81005859375</v>
+        <v>347.7099609375</v>
       </c>
       <c r="I2">
-        <v>56.79931640625</v>
+        <v>49.4794921875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1623,10 +1623,10 @@
         <v>42</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>443.6298828125</v>
+        <v>374.509765625</v>
       </c>
       <c r="H3">
-        <v>422.739990234375</v>
+        <v>366.6298828125</v>
       </c>
       <c r="I3">
-        <v>20.889892578125</v>
+        <v>7.8798828125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1664,16 +1664,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4">
-        <v>456.26025390625</v>
+        <v>394.16015625</v>
       </c>
       <c r="H4">
-        <v>457.349609375</v>
+        <v>387.9296875</v>
       </c>
       <c r="I4">
-        <v>-1.08935546875</v>
+        <v>6.23046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>401.940185546875</v>
+        <v>345.830078125</v>
       </c>
       <c r="H5">
-        <v>478.5400390625</v>
+        <v>409.419921875</v>
       </c>
       <c r="I5">
-        <v>-76.599853515625</v>
+        <v>-63.58984375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1770,16 +1770,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>497.169921875</v>
+        <v>403.77978515625</v>
       </c>
       <c r="H2">
-        <v>492.31005859375</v>
+        <v>374.259765625</v>
       </c>
       <c r="I2">
-        <v>4.85986328125</v>
+        <v>29.52001953125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>481.18994140625</v>
+        <v>358.079833984375</v>
       </c>
       <c r="H3">
-        <v>457.259765625</v>
+        <v>375.47021484375</v>
       </c>
       <c r="I3">
-        <v>23.93017578125</v>
+        <v>-17.390380859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1825,10 +1825,10 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1837,13 +1837,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>470.1796875</v>
+        <v>414.169921875</v>
       </c>
       <c r="H4">
-        <v>468.0693359375</v>
+        <v>414.89990234375</v>
       </c>
       <c r="I4">
-        <v>2.1103515625</v>
+        <v>-0.72998046875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1857,10 +1857,10 @@
         <v>49</v>
       </c>
       <c r="C5">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1869,13 +1869,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>410.27978515625</v>
+        <v>404.4697265625</v>
       </c>
       <c r="H5">
-        <v>441.18017578125</v>
+        <v>415.869384765625</v>
       </c>
       <c r="I5">
-        <v>-30.900390625</v>
+        <v>-11.399658203125</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>

<commit_message>
Ajusta oitavas da Sul-Americana e corrige fase 1 da Libertadores
</commit_message>
<xml_diff>
--- a/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
+++ b/libertadores/datasets_liberta/classificacao_por_grupo_fase_1.xlsx
@@ -77,12 +77,12 @@
     <t>LISI GREMISTA</t>
   </si>
   <si>
+    <t>Máquina Laranjja</t>
+  </si>
+  <si>
     <t>S.E.R. GRILLO</t>
   </si>
   <si>
-    <t>Máquina Laranjja</t>
-  </si>
-  <si>
     <t>Grupo C</t>
   </si>
   <si>
@@ -104,15 +104,15 @@
     <t>A Lenda Super Vasco F.c</t>
   </si>
   <si>
+    <t>Mau Humor F.C.</t>
+  </si>
+  <si>
+    <t>Grêmio imortal 36</t>
+  </si>
+  <si>
     <t>FBC Colorado</t>
   </si>
   <si>
-    <t>Mau Humor F.C.</t>
-  </si>
-  <si>
-    <t>Grêmio imortal 36</t>
-  </si>
-  <si>
     <t>Grupo E</t>
   </si>
   <si>
@@ -134,12 +134,12 @@
     <t>lsauer fc</t>
   </si>
   <si>
+    <t>DM Studio</t>
+  </si>
+  <si>
     <t>AZURRA82</t>
   </si>
   <si>
-    <t>DM Studio</t>
-  </si>
-  <si>
     <t>Rolo Compressor ZN</t>
   </si>
   <si>
@@ -161,16 +161,16 @@
     <t>Grupo H</t>
   </si>
   <si>
+    <t>Texas Club 2026</t>
+  </si>
+  <si>
     <t>TEAM LOPES 99</t>
   </si>
   <si>
+    <t>Super Vasco f.c</t>
+  </si>
+  <si>
     <t>Gremiomaniasm</t>
-  </si>
-  <si>
-    <t>Texas Club 2026</t>
-  </si>
-  <si>
-    <t>Super Vasco f.c</t>
   </si>
 </sst>
 </file>
@@ -571,10 +571,10 @@
         <v>11</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -583,13 +583,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>383.909912109375</v>
+        <v>445.919921875</v>
       </c>
       <c r="H2">
-        <v>340.740234375</v>
+        <v>388.940185546875</v>
       </c>
       <c r="I2">
-        <v>43.169677734375</v>
+        <v>56.979736328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -603,10 +603,10 @@
         <v>12</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -615,13 +615,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>364.060302734375</v>
+        <v>426.980224609375</v>
       </c>
       <c r="H3">
-        <v>303.0997314453125</v>
+        <v>357.3096923828125</v>
       </c>
       <c r="I3">
-        <v>60.9605712890625</v>
+        <v>69.6705322265625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -644,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>343.10986328125</v>
+        <v>397.31982421875</v>
       </c>
       <c r="H4">
-        <v>358.4501953125</v>
+        <v>421.3701171875</v>
       </c>
       <c r="I4">
-        <v>-15.34033203125</v>
+        <v>-24.05029296875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -676,16 +676,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>253.0401611328125</v>
+        <v>301.2401123046875</v>
       </c>
       <c r="H5">
-        <v>341.830078125</v>
+        <v>403.840087890625</v>
       </c>
       <c r="I5">
-        <v>-88.7899169921875</v>
+        <v>-102.5999755859375</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -753,13 +753,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>406.02001953125</v>
+        <v>478.1298828125</v>
       </c>
       <c r="H2">
-        <v>333.770263671875</v>
+        <v>398.130126953125</v>
       </c>
       <c r="I2">
-        <v>72.249755859375</v>
+        <v>79.999755859375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -782,16 +782,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>383.469482421875</v>
+        <v>447.829345703125</v>
       </c>
       <c r="H3">
-        <v>384.60009765625</v>
+        <v>456.7099609375</v>
       </c>
       <c r="I3">
-        <v>-1.130615234375</v>
+        <v>-8.880615234375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -814,16 +814,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>361.580078125</v>
+        <v>434.969970703125</v>
       </c>
       <c r="H4">
-        <v>371.899658203125</v>
+        <v>476.159423828125</v>
       </c>
       <c r="I4">
-        <v>-10.319580078125</v>
+        <v>-41.189453125</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -837,10 +837,10 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -849,13 +849,13 @@
         <v>4</v>
       </c>
       <c r="G5">
-        <v>370.849853515625</v>
+        <v>406.090087890625</v>
       </c>
       <c r="H5">
-        <v>431.6494140625</v>
+        <v>436.019775390625</v>
       </c>
       <c r="I5">
-        <v>-60.799560546875</v>
+        <v>-29.9296875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -911,10 +911,10 @@
         <v>21</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>440.9697265625</v>
+        <v>527.3896484375</v>
       </c>
       <c r="H2">
-        <v>373.98974609375</v>
+        <v>456.98974609375</v>
       </c>
       <c r="I2">
-        <v>66.97998046875</v>
+        <v>70.39990234375</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>407.669921875</v>
+        <v>490.669921875</v>
       </c>
       <c r="H3">
-        <v>411.31005859375</v>
+        <v>497.72998046875</v>
       </c>
       <c r="I3">
-        <v>-3.64013671875</v>
+        <v>-7.06005859375</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -975,10 +975,10 @@
         <v>23</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -987,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>377.9794921875</v>
+        <v>444.58935546875</v>
       </c>
       <c r="H4">
-        <v>427.669677734375</v>
+        <v>484.069580078125</v>
       </c>
       <c r="I4">
-        <v>-49.690185546875</v>
+        <v>-39.480224609375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1016,16 +1016,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>404.719970703125</v>
+        <v>461.119873046875</v>
       </c>
       <c r="H5">
-        <v>418.36962890625</v>
+        <v>484.9794921875</v>
       </c>
       <c r="I5">
-        <v>-13.649658203125</v>
+        <v>-23.859619140625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1090,16 +1090,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>373.920166015625</v>
+        <v>442.719970703125</v>
       </c>
       <c r="H2">
-        <v>376.52978515625</v>
+        <v>448.61962890625</v>
       </c>
       <c r="I2">
-        <v>-2.609619140625</v>
+        <v>-5.899658203125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1113,10 +1113,10 @@
         <v>27</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1125,13 +1125,13 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>387.249755859375</v>
+        <v>439.99951171875</v>
       </c>
       <c r="H3">
-        <v>370.39990234375</v>
+        <v>408.960205078125</v>
       </c>
       <c r="I3">
-        <v>16.849853515625</v>
+        <v>31.039306640625</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1145,10 +1145,10 @@
         <v>28</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1157,13 +1157,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>385.189453125</v>
+        <v>435.2802734375</v>
       </c>
       <c r="H4">
-        <v>361.5703125</v>
+        <v>469.849609375</v>
       </c>
       <c r="I4">
-        <v>23.619140625</v>
+        <v>-34.5693359375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1186,16 +1186,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>363.1904296875</v>
+        <v>434.6396484375</v>
       </c>
       <c r="H5">
-        <v>401.0498046875</v>
+        <v>425.2099609375</v>
       </c>
       <c r="I5">
-        <v>-37.859375</v>
+        <v>9.4296875</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1251,10 +1251,10 @@
         <v>31</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1263,13 +1263,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>411.74951171875</v>
+        <v>474.5595703125</v>
       </c>
       <c r="H2">
-        <v>397.419921875</v>
+        <v>450.8798828125</v>
       </c>
       <c r="I2">
-        <v>14.32958984375</v>
+        <v>23.6796875</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1292,16 +1292,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>419.9599609375</v>
+        <v>485.85009765625</v>
       </c>
       <c r="H3">
-        <v>388.109619140625</v>
+        <v>461.329833984375</v>
       </c>
       <c r="I3">
-        <v>31.850341796875</v>
+        <v>24.520263671875</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1327,13 +1327,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>376.389892578125</v>
+        <v>449.610107421875</v>
       </c>
       <c r="H4">
-        <v>368.1298828125</v>
+        <v>434.02001953125</v>
       </c>
       <c r="I4">
-        <v>8.260009765625</v>
+        <v>15.590087890625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>366.03955078125</v>
+        <v>419.49951171875</v>
       </c>
       <c r="H5">
-        <v>420.4794921875</v>
+        <v>483.28955078125</v>
       </c>
       <c r="I5">
-        <v>-54.43994140625</v>
+        <v>-63.7900390625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1421,10 +1421,10 @@
         <v>36</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>413.60009765625</v>
+        <v>472.210205078125</v>
       </c>
       <c r="H2">
-        <v>365.769775390625</v>
+        <v>420.389892578125</v>
       </c>
       <c r="I2">
-        <v>47.830322265625</v>
+        <v>51.8203125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1462,16 +1462,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>370.239990234375</v>
+        <v>436.039794921875</v>
       </c>
       <c r="H3">
-        <v>337.939697265625</v>
+        <v>453</v>
       </c>
       <c r="I3">
-        <v>32.30029296875</v>
+        <v>-16.960205078125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1485,10 +1485,10 @@
         <v>38</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1497,13 +1497,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>368.849853515625</v>
+        <v>424.860107421875</v>
       </c>
       <c r="H4">
-        <v>386.490234375</v>
+        <v>396.5498046875</v>
       </c>
       <c r="I4">
-        <v>-17.640380859375</v>
+        <v>28.310302734375</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1526,16 +1526,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>353.489501953125</v>
+        <v>419.999267578125</v>
       </c>
       <c r="H5">
-        <v>415.979736328125</v>
+        <v>483.169677734375</v>
       </c>
       <c r="I5">
-        <v>-62.490234375</v>
+        <v>-63.17041015625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1591,10 +1591,10 @@
         <v>41</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1603,13 +1603,13 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <v>397.189453125</v>
+        <v>466.609375</v>
       </c>
       <c r="H2">
-        <v>347.7099609375</v>
+        <v>409.81005859375</v>
       </c>
       <c r="I2">
-        <v>49.4794921875</v>
+        <v>56.79931640625</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1623,10 +1623,10 @@
         <v>42</v>
       </c>
       <c r="C3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1635,13 +1635,13 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>374.509765625</v>
+        <v>443.6298828125</v>
       </c>
       <c r="H3">
-        <v>366.6298828125</v>
+        <v>422.739990234375</v>
       </c>
       <c r="I3">
-        <v>7.8798828125</v>
+        <v>20.889892578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1664,16 +1664,16 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>394.16015625</v>
+        <v>456.26025390625</v>
       </c>
       <c r="H4">
-        <v>387.9296875</v>
+        <v>457.349609375</v>
       </c>
       <c r="I4">
-        <v>6.23046875</v>
+        <v>-1.08935546875</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1696,16 +1696,16 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>345.830078125</v>
+        <v>401.940185546875</v>
       </c>
       <c r="H5">
-        <v>409.419921875</v>
+        <v>478.5400390625</v>
       </c>
       <c r="I5">
-        <v>-63.58984375</v>
+        <v>-76.599853515625</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1770,16 +1770,16 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>403.77978515625</v>
+        <v>497.169921875</v>
       </c>
       <c r="H2">
-        <v>374.259765625</v>
+        <v>492.31005859375</v>
       </c>
       <c r="I2">
-        <v>29.52001953125</v>
+        <v>4.85986328125</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>358.079833984375</v>
+        <v>481.18994140625</v>
       </c>
       <c r="H3">
-        <v>375.47021484375</v>
+        <v>457.259765625</v>
       </c>
       <c r="I3">
-        <v>-17.390380859375</v>
+        <v>23.93017578125</v>
       </c>
       <c r="J3">
         <v>2</v>
@@ -1825,10 +1825,10 @@
         <v>48</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1837,13 +1837,13 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>414.169921875</v>
+        <v>470.1796875</v>
       </c>
       <c r="H4">
-        <v>414.89990234375</v>
+        <v>468.0693359375</v>
       </c>
       <c r="I4">
-        <v>-0.72998046875</v>
+        <v>2.1103515625</v>
       </c>
       <c r="J4">
         <v>3</v>
@@ -1857,10 +1857,10 @@
         <v>49</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1869,13 +1869,13 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>404.4697265625</v>
+        <v>410.27978515625</v>
       </c>
       <c r="H5">
-        <v>415.869384765625</v>
+        <v>441.18017578125</v>
       </c>
       <c r="I5">
-        <v>-11.399658203125</v>
+        <v>-30.900390625</v>
       </c>
       <c r="J5">
         <v>4</v>

</xml_diff>